<commit_message>
Remove status and update comments in immunization profile
Remove status field and update comments in FRCoreImmunizationProfile.fsh

Réu du 22 juin 54e27aaeb16b9f6dd05dc9aede8b30f0842204f3
</commit_message>
<xml_diff>
--- a/nr-doc-core-immunization/ig/StructureDefinition-fr-core-immunization.xlsx
+++ b/nr-doc-core-immunization/ig/StructureDefinition-fr-core-immunization.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5311" uniqueCount="679">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5311" uniqueCount="678">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-22T13:09:12+00:00</t>
+    <t>2026-06-22T13:13:25+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -882,9 +882,6 @@
   </si>
   <si>
     <t>Will generally be set to show that the immunization has been completed or not done.  This element is labeled as a modifier because the status contains codes that mark the resource as not currently valid.</t>
-  </si>
-  <si>
-    <t>completed</t>
   </si>
   <si>
     <t>required</t>
@@ -9159,28 +9156,28 @@
         <v>79</v>
       </c>
       <c r="S58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="T58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="U58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="V58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="W58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="X58" t="s" s="2">
         <v>278</v>
       </c>
-      <c r="T58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X58" t="s" s="2">
+      <c r="Y58" t="s" s="2">
         <v>279</v>
       </c>
-      <c r="Y58" t="s" s="2">
+      <c r="Z58" t="s" s="2">
         <v>280</v>
-      </c>
-      <c r="Z58" t="s" s="2">
-        <v>281</v>
       </c>
       <c r="AA58" t="s" s="2">
         <v>79</v>
@@ -9213,16 +9210,16 @@
         <v>102</v>
       </c>
       <c r="AK58" t="s" s="2">
+        <v>281</v>
+      </c>
+      <c r="AL58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM58" t="s" s="2">
         <v>282</v>
       </c>
-      <c r="AL58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM58" t="s" s="2">
+      <c r="AN58" t="s" s="2">
         <v>283</v>
-      </c>
-      <c r="AN58" t="s" s="2">
-        <v>284</v>
       </c>
       <c r="AO58" t="s" s="2">
         <v>79</v>
@@ -9230,10 +9227,10 @@
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -9259,13 +9256,13 @@
         <v>195</v>
       </c>
       <c r="L59" t="s" s="2">
+        <v>285</v>
+      </c>
+      <c r="M59" t="s" s="2">
         <v>286</v>
       </c>
-      <c r="M59" t="s" s="2">
+      <c r="N59" t="s" s="2">
         <v>287</v>
-      </c>
-      <c r="N59" t="s" s="2">
-        <v>288</v>
       </c>
       <c r="O59" s="2"/>
       <c r="P59" t="s" s="2">
@@ -9291,14 +9288,14 @@
         <v>79</v>
       </c>
       <c r="X59" t="s" s="2">
+        <v>288</v>
+      </c>
+      <c r="Y59" t="s" s="2">
         <v>289</v>
       </c>
-      <c r="Y59" t="s" s="2">
+      <c r="Z59" t="s" s="2">
         <v>290</v>
       </c>
-      <c r="Z59" t="s" s="2">
-        <v>291</v>
-      </c>
       <c r="AA59" t="s" s="2">
         <v>79</v>
       </c>
@@ -9315,7 +9312,7 @@
         <v>79</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>80</v>
@@ -9330,13 +9327,13 @@
         <v>102</v>
       </c>
       <c r="AK59" t="s" s="2">
+        <v>291</v>
+      </c>
+      <c r="AL59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM59" t="s" s="2">
         <v>292</v>
-      </c>
-      <c r="AL59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM59" t="s" s="2">
-        <v>293</v>
       </c>
       <c r="AN59" t="s" s="2">
         <v>79</v>
@@ -9347,10 +9344,10 @@
     </row>
     <row r="60">
       <c r="A60" t="s" s="2">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -9376,10 +9373,10 @@
         <v>195</v>
       </c>
       <c r="L60" t="s" s="2">
+        <v>294</v>
+      </c>
+      <c r="M60" t="s" s="2">
         <v>295</v>
-      </c>
-      <c r="M60" t="s" s="2">
-        <v>296</v>
       </c>
       <c r="N60" s="2"/>
       <c r="O60" s="2"/>
@@ -9409,11 +9406,11 @@
         <v>114</v>
       </c>
       <c r="Y60" t="s" s="2">
+        <v>296</v>
+      </c>
+      <c r="Z60" t="s" s="2">
         <v>297</v>
       </c>
-      <c r="Z60" t="s" s="2">
-        <v>298</v>
-      </c>
       <c r="AA60" t="s" s="2">
         <v>79</v>
       </c>
@@ -9430,7 +9427,7 @@
         <v>79</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>90</v>
@@ -9445,27 +9442,27 @@
         <v>102</v>
       </c>
       <c r="AK60" t="s" s="2">
+        <v>298</v>
+      </c>
+      <c r="AL60" t="s" s="2">
         <v>299</v>
       </c>
-      <c r="AL60" t="s" s="2">
+      <c r="AM60" t="s" s="2">
         <v>300</v>
       </c>
-      <c r="AM60" t="s" s="2">
+      <c r="AN60" t="s" s="2">
         <v>301</v>
       </c>
-      <c r="AN60" t="s" s="2">
+      <c r="AO60" t="s" s="2">
         <v>302</v>
-      </c>
-      <c r="AO60" t="s" s="2">
-        <v>303</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="2">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -9577,10 +9574,10 @@
     </row>
     <row r="62">
       <c r="A62" t="s" s="2">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -9694,10 +9691,10 @@
     </row>
     <row r="63">
       <c r="A63" t="s" s="2">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -9720,19 +9717,19 @@
         <v>91</v>
       </c>
       <c r="K63" t="s" s="2">
+        <v>306</v>
+      </c>
+      <c r="L63" t="s" s="2">
         <v>307</v>
       </c>
-      <c r="L63" t="s" s="2">
+      <c r="M63" t="s" s="2">
         <v>308</v>
       </c>
-      <c r="M63" t="s" s="2">
+      <c r="N63" t="s" s="2">
         <v>309</v>
       </c>
-      <c r="N63" t="s" s="2">
+      <c r="O63" t="s" s="2">
         <v>310</v>
-      </c>
-      <c r="O63" t="s" s="2">
-        <v>311</v>
       </c>
       <c r="P63" t="s" s="2">
         <v>79</v>
@@ -9769,10 +9766,10 @@
         <v>79</v>
       </c>
       <c r="AB63" t="s" s="2">
+        <v>311</v>
+      </c>
+      <c r="AC63" t="s" s="2">
         <v>312</v>
-      </c>
-      <c r="AC63" t="s" s="2">
-        <v>313</v>
       </c>
       <c r="AD63" t="s" s="2">
         <v>79</v>
@@ -9781,7 +9778,7 @@
         <v>139</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>80</v>
@@ -9799,10 +9796,10 @@
         <v>79</v>
       </c>
       <c r="AL63" t="s" s="2">
+        <v>314</v>
+      </c>
+      <c r="AM63" t="s" s="2">
         <v>315</v>
-      </c>
-      <c r="AM63" t="s" s="2">
-        <v>316</v>
       </c>
       <c r="AN63" t="s" s="2">
         <v>79</v>
@@ -9813,13 +9810,13 @@
     </row>
     <row r="64">
       <c r="A64" t="s" s="2">
+        <v>316</v>
+      </c>
+      <c r="B64" t="s" s="2">
+        <v>305</v>
+      </c>
+      <c r="C64" t="s" s="2">
         <v>317</v>
-      </c>
-      <c r="B64" t="s" s="2">
-        <v>306</v>
-      </c>
-      <c r="C64" t="s" s="2">
-        <v>318</v>
       </c>
       <c r="D64" t="s" s="2">
         <v>79</v>
@@ -9841,19 +9838,19 @@
         <v>91</v>
       </c>
       <c r="K64" t="s" s="2">
+        <v>306</v>
+      </c>
+      <c r="L64" t="s" s="2">
         <v>307</v>
       </c>
-      <c r="L64" t="s" s="2">
+      <c r="M64" t="s" s="2">
         <v>308</v>
       </c>
-      <c r="M64" t="s" s="2">
+      <c r="N64" t="s" s="2">
         <v>309</v>
       </c>
-      <c r="N64" t="s" s="2">
+      <c r="O64" t="s" s="2">
         <v>310</v>
-      </c>
-      <c r="O64" t="s" s="2">
-        <v>311</v>
       </c>
       <c r="P64" t="s" s="2">
         <v>79</v>
@@ -9878,11 +9875,11 @@
         <v>79</v>
       </c>
       <c r="X64" t="s" s="2">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="Y64" s="2"/>
       <c r="Z64" t="s" s="2">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="AA64" t="s" s="2">
         <v>79</v>
@@ -9900,7 +9897,7 @@
         <v>79</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>80</v>
@@ -9918,10 +9915,10 @@
         <v>79</v>
       </c>
       <c r="AL64" t="s" s="2">
+        <v>314</v>
+      </c>
+      <c r="AM64" t="s" s="2">
         <v>315</v>
-      </c>
-      <c r="AM64" t="s" s="2">
-        <v>316</v>
       </c>
       <c r="AN64" t="s" s="2">
         <v>79</v>
@@ -9932,13 +9929,13 @@
     </row>
     <row r="65">
       <c r="A65" t="s" s="2">
+        <v>319</v>
+      </c>
+      <c r="B65" t="s" s="2">
+        <v>305</v>
+      </c>
+      <c r="C65" t="s" s="2">
         <v>320</v>
-      </c>
-      <c r="B65" t="s" s="2">
-        <v>306</v>
-      </c>
-      <c r="C65" t="s" s="2">
-        <v>321</v>
       </c>
       <c r="D65" t="s" s="2">
         <v>79</v>
@@ -9960,19 +9957,19 @@
         <v>91</v>
       </c>
       <c r="K65" t="s" s="2">
+        <v>306</v>
+      </c>
+      <c r="L65" t="s" s="2">
         <v>307</v>
       </c>
-      <c r="L65" t="s" s="2">
+      <c r="M65" t="s" s="2">
         <v>308</v>
       </c>
-      <c r="M65" t="s" s="2">
+      <c r="N65" t="s" s="2">
         <v>309</v>
       </c>
-      <c r="N65" t="s" s="2">
+      <c r="O65" t="s" s="2">
         <v>310</v>
-      </c>
-      <c r="O65" t="s" s="2">
-        <v>311</v>
       </c>
       <c r="P65" t="s" s="2">
         <v>79</v>
@@ -9997,11 +9994,11 @@
         <v>79</v>
       </c>
       <c r="X65" t="s" s="2">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="Y65" s="2"/>
       <c r="Z65" t="s" s="2">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="AA65" t="s" s="2">
         <v>79</v>
@@ -10019,7 +10016,7 @@
         <v>79</v>
       </c>
       <c r="AF65" t="s" s="2">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="AG65" t="s" s="2">
         <v>80</v>
@@ -10037,10 +10034,10 @@
         <v>79</v>
       </c>
       <c r="AL65" t="s" s="2">
+        <v>314</v>
+      </c>
+      <c r="AM65" t="s" s="2">
         <v>315</v>
-      </c>
-      <c r="AM65" t="s" s="2">
-        <v>316</v>
       </c>
       <c r="AN65" t="s" s="2">
         <v>79</v>
@@ -10051,10 +10048,10 @@
     </row>
     <row r="66">
       <c r="A66" t="s" s="2">
+        <v>322</v>
+      </c>
+      <c r="B66" t="s" s="2">
         <v>323</v>
-      </c>
-      <c r="B66" t="s" s="2">
-        <v>324</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
@@ -10166,10 +10163,10 @@
     </row>
     <row r="67">
       <c r="A67" t="s" s="2">
+        <v>324</v>
+      </c>
+      <c r="B67" t="s" s="2">
         <v>325</v>
-      </c>
-      <c r="B67" t="s" s="2">
-        <v>326</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -10283,10 +10280,10 @@
     </row>
     <row r="68">
       <c r="A68" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="B68" t="s" s="2">
         <v>327</v>
-      </c>
-      <c r="B68" t="s" s="2">
-        <v>328</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -10312,16 +10309,16 @@
         <v>104</v>
       </c>
       <c r="L68" t="s" s="2">
+        <v>328</v>
+      </c>
+      <c r="M68" t="s" s="2">
         <v>329</v>
       </c>
-      <c r="M68" t="s" s="2">
+      <c r="N68" t="s" s="2">
         <v>330</v>
       </c>
-      <c r="N68" t="s" s="2">
+      <c r="O68" t="s" s="2">
         <v>331</v>
-      </c>
-      <c r="O68" t="s" s="2">
-        <v>332</v>
       </c>
       <c r="P68" t="s" s="2">
         <v>79</v>
@@ -10370,7 +10367,7 @@
         <v>79</v>
       </c>
       <c r="AF68" t="s" s="2">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="AG68" t="s" s="2">
         <v>80</v>
@@ -10388,10 +10385,10 @@
         <v>79</v>
       </c>
       <c r="AL68" t="s" s="2">
+        <v>333</v>
+      </c>
+      <c r="AM68" t="s" s="2">
         <v>334</v>
-      </c>
-      <c r="AM68" t="s" s="2">
-        <v>335</v>
       </c>
       <c r="AN68" t="s" s="2">
         <v>79</v>
@@ -10402,10 +10399,10 @@
     </row>
     <row r="69">
       <c r="A69" t="s" s="2">
+        <v>335</v>
+      </c>
+      <c r="B69" t="s" s="2">
         <v>336</v>
-      </c>
-      <c r="B69" t="s" s="2">
-        <v>337</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -10431,13 +10428,13 @@
         <v>151</v>
       </c>
       <c r="L69" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="M69" t="s" s="2">
         <v>338</v>
       </c>
-      <c r="M69" t="s" s="2">
+      <c r="N69" t="s" s="2">
         <v>339</v>
-      </c>
-      <c r="N69" t="s" s="2">
-        <v>340</v>
       </c>
       <c r="O69" s="2"/>
       <c r="P69" t="s" s="2">
@@ -10487,7 +10484,7 @@
         <v>79</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="AG69" t="s" s="2">
         <v>80</v>
@@ -10505,10 +10502,10 @@
         <v>79</v>
       </c>
       <c r="AL69" t="s" s="2">
+        <v>341</v>
+      </c>
+      <c r="AM69" t="s" s="2">
         <v>342</v>
-      </c>
-      <c r="AM69" t="s" s="2">
-        <v>343</v>
       </c>
       <c r="AN69" t="s" s="2">
         <v>79</v>
@@ -10519,10 +10516,10 @@
     </row>
     <row r="70">
       <c r="A70" t="s" s="2">
+        <v>343</v>
+      </c>
+      <c r="B70" t="s" s="2">
         <v>344</v>
-      </c>
-      <c r="B70" t="s" s="2">
-        <v>345</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -10548,14 +10545,14 @@
         <v>110</v>
       </c>
       <c r="L70" t="s" s="2">
+        <v>345</v>
+      </c>
+      <c r="M70" t="s" s="2">
         <v>346</v>
-      </c>
-      <c r="M70" t="s" s="2">
-        <v>347</v>
       </c>
       <c r="N70" s="2"/>
       <c r="O70" t="s" s="2">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="P70" t="s" s="2">
         <v>79</v>
@@ -10604,7 +10601,7 @@
         <v>79</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>80</v>
@@ -10622,10 +10619,10 @@
         <v>79</v>
       </c>
       <c r="AL70" t="s" s="2">
+        <v>349</v>
+      </c>
+      <c r="AM70" t="s" s="2">
         <v>350</v>
-      </c>
-      <c r="AM70" t="s" s="2">
-        <v>351</v>
       </c>
       <c r="AN70" t="s" s="2">
         <v>79</v>
@@ -10636,10 +10633,10 @@
     </row>
     <row r="71">
       <c r="A71" t="s" s="2">
+        <v>351</v>
+      </c>
+      <c r="B71" t="s" s="2">
         <v>352</v>
-      </c>
-      <c r="B71" t="s" s="2">
-        <v>353</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
@@ -10665,14 +10662,14 @@
         <v>151</v>
       </c>
       <c r="L71" t="s" s="2">
+        <v>353</v>
+      </c>
+      <c r="M71" t="s" s="2">
         <v>354</v>
-      </c>
-      <c r="M71" t="s" s="2">
-        <v>355</v>
       </c>
       <c r="N71" s="2"/>
       <c r="O71" t="s" s="2">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="P71" t="s" s="2">
         <v>79</v>
@@ -10721,7 +10718,7 @@
         <v>79</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>80</v>
@@ -10739,10 +10736,10 @@
         <v>79</v>
       </c>
       <c r="AL71" t="s" s="2">
+        <v>357</v>
+      </c>
+      <c r="AM71" t="s" s="2">
         <v>358</v>
-      </c>
-      <c r="AM71" t="s" s="2">
-        <v>359</v>
       </c>
       <c r="AN71" t="s" s="2">
         <v>79</v>
@@ -10753,10 +10750,10 @@
     </row>
     <row r="72">
       <c r="A72" t="s" s="2">
+        <v>359</v>
+      </c>
+      <c r="B72" t="s" s="2">
         <v>360</v>
-      </c>
-      <c r="B72" t="s" s="2">
-        <v>361</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -10779,19 +10776,19 @@
         <v>91</v>
       </c>
       <c r="K72" t="s" s="2">
+        <v>361</v>
+      </c>
+      <c r="L72" t="s" s="2">
         <v>362</v>
       </c>
-      <c r="L72" t="s" s="2">
+      <c r="M72" t="s" s="2">
         <v>363</v>
       </c>
-      <c r="M72" t="s" s="2">
+      <c r="N72" t="s" s="2">
         <v>364</v>
       </c>
-      <c r="N72" t="s" s="2">
+      <c r="O72" t="s" s="2">
         <v>365</v>
-      </c>
-      <c r="O72" t="s" s="2">
-        <v>366</v>
       </c>
       <c r="P72" t="s" s="2">
         <v>79</v>
@@ -10840,7 +10837,7 @@
         <v>79</v>
       </c>
       <c r="AF72" t="s" s="2">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="AG72" t="s" s="2">
         <v>80</v>
@@ -10858,10 +10855,10 @@
         <v>79</v>
       </c>
       <c r="AL72" t="s" s="2">
+        <v>367</v>
+      </c>
+      <c r="AM72" t="s" s="2">
         <v>368</v>
-      </c>
-      <c r="AM72" t="s" s="2">
-        <v>369</v>
       </c>
       <c r="AN72" t="s" s="2">
         <v>79</v>
@@ -10872,10 +10869,10 @@
     </row>
     <row r="73">
       <c r="A73" t="s" s="2">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -10901,16 +10898,16 @@
         <v>151</v>
       </c>
       <c r="L73" t="s" s="2">
+        <v>370</v>
+      </c>
+      <c r="M73" t="s" s="2">
         <v>371</v>
       </c>
-      <c r="M73" t="s" s="2">
+      <c r="N73" t="s" s="2">
         <v>372</v>
       </c>
-      <c r="N73" t="s" s="2">
+      <c r="O73" t="s" s="2">
         <v>373</v>
-      </c>
-      <c r="O73" t="s" s="2">
-        <v>374</v>
       </c>
       <c r="P73" t="s" s="2">
         <v>79</v>
@@ -10959,7 +10956,7 @@
         <v>79</v>
       </c>
       <c r="AF73" t="s" s="2">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="AG73" t="s" s="2">
         <v>80</v>
@@ -10977,10 +10974,10 @@
         <v>79</v>
       </c>
       <c r="AL73" t="s" s="2">
+        <v>375</v>
+      </c>
+      <c r="AM73" t="s" s="2">
         <v>376</v>
-      </c>
-      <c r="AM73" t="s" s="2">
-        <v>377</v>
       </c>
       <c r="AN73" t="s" s="2">
         <v>79</v>
@@ -10991,10 +10988,10 @@
     </row>
     <row r="74">
       <c r="A74" t="s" s="2">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
@@ -11017,13 +11014,13 @@
         <v>91</v>
       </c>
       <c r="K74" t="s" s="2">
+        <v>378</v>
+      </c>
+      <c r="L74" t="s" s="2">
         <v>379</v>
       </c>
-      <c r="L74" t="s" s="2">
+      <c r="M74" t="s" s="2">
         <v>380</v>
-      </c>
-      <c r="M74" t="s" s="2">
-        <v>381</v>
       </c>
       <c r="N74" s="2"/>
       <c r="O74" s="2"/>
@@ -11074,7 +11071,7 @@
         <v>79</v>
       </c>
       <c r="AF74" t="s" s="2">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="AG74" t="s" s="2">
         <v>90</v>
@@ -11089,16 +11086,16 @@
         <v>102</v>
       </c>
       <c r="AK74" t="s" s="2">
+        <v>381</v>
+      </c>
+      <c r="AL74" t="s" s="2">
         <v>382</v>
       </c>
-      <c r="AL74" t="s" s="2">
+      <c r="AM74" t="s" s="2">
         <v>383</v>
       </c>
-      <c r="AM74" t="s" s="2">
+      <c r="AN74" t="s" s="2">
         <v>384</v>
-      </c>
-      <c r="AN74" t="s" s="2">
-        <v>385</v>
       </c>
       <c r="AO74" t="s" s="2">
         <v>79</v>
@@ -11106,10 +11103,10 @@
     </row>
     <row r="75">
       <c r="A75" t="s" s="2">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
@@ -11132,13 +11129,13 @@
         <v>79</v>
       </c>
       <c r="K75" t="s" s="2">
+        <v>386</v>
+      </c>
+      <c r="L75" t="s" s="2">
         <v>387</v>
       </c>
-      <c r="L75" t="s" s="2">
+      <c r="M75" t="s" s="2">
         <v>388</v>
-      </c>
-      <c r="M75" t="s" s="2">
-        <v>389</v>
       </c>
       <c r="N75" s="2"/>
       <c r="O75" s="2"/>
@@ -11189,7 +11186,7 @@
         <v>79</v>
       </c>
       <c r="AF75" t="s" s="2">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="AG75" t="s" s="2">
         <v>80</v>
@@ -11204,16 +11201,16 @@
         <v>102</v>
       </c>
       <c r="AK75" t="s" s="2">
+        <v>389</v>
+      </c>
+      <c r="AL75" t="s" s="2">
         <v>390</v>
       </c>
-      <c r="AL75" t="s" s="2">
+      <c r="AM75" t="s" s="2">
         <v>391</v>
       </c>
-      <c r="AM75" t="s" s="2">
+      <c r="AN75" t="s" s="2">
         <v>392</v>
-      </c>
-      <c r="AN75" t="s" s="2">
-        <v>393</v>
       </c>
       <c r="AO75" t="s" s="2">
         <v>79</v>
@@ -11221,10 +11218,10 @@
     </row>
     <row r="76">
       <c r="A76" t="s" s="2">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -11247,16 +11244,16 @@
         <v>91</v>
       </c>
       <c r="K76" t="s" s="2">
+        <v>394</v>
+      </c>
+      <c r="L76" t="s" s="2">
         <v>395</v>
       </c>
-      <c r="L76" t="s" s="2">
+      <c r="M76" t="s" s="2">
         <v>396</v>
       </c>
-      <c r="M76" t="s" s="2">
+      <c r="N76" t="s" s="2">
         <v>397</v>
-      </c>
-      <c r="N76" t="s" s="2">
-        <v>398</v>
       </c>
       <c r="O76" s="2"/>
       <c r="P76" t="s" s="2">
@@ -11294,17 +11291,17 @@
         <v>79</v>
       </c>
       <c r="AB76" t="s" s="2">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="AC76" s="2"/>
       <c r="AD76" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE76" t="s" s="2">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="AF76" t="s" s="2">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="AG76" t="s" s="2">
         <v>90</v>
@@ -11319,30 +11316,30 @@
         <v>102</v>
       </c>
       <c r="AK76" t="s" s="2">
+        <v>400</v>
+      </c>
+      <c r="AL76" t="s" s="2">
         <v>401</v>
       </c>
-      <c r="AL76" t="s" s="2">
+      <c r="AM76" t="s" s="2">
         <v>402</v>
       </c>
-      <c r="AM76" t="s" s="2">
+      <c r="AN76" t="s" s="2">
         <v>403</v>
       </c>
-      <c r="AN76" t="s" s="2">
+      <c r="AO76" t="s" s="2">
         <v>404</v>
-      </c>
-      <c r="AO76" t="s" s="2">
-        <v>405</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s" s="2">
+        <v>405</v>
+      </c>
+      <c r="B77" t="s" s="2">
+        <v>393</v>
+      </c>
+      <c r="C77" t="s" s="2">
         <v>406</v>
-      </c>
-      <c r="B77" t="s" s="2">
-        <v>394</v>
-      </c>
-      <c r="C77" t="s" s="2">
-        <v>407</v>
       </c>
       <c r="D77" t="s" s="2">
         <v>79</v>
@@ -11364,16 +11361,16 @@
         <v>91</v>
       </c>
       <c r="K77" t="s" s="2">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="L77" t="s" s="2">
+        <v>407</v>
+      </c>
+      <c r="M77" t="s" s="2">
         <v>408</v>
       </c>
-      <c r="M77" t="s" s="2">
-        <v>409</v>
-      </c>
       <c r="N77" t="s" s="2">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="O77" s="2"/>
       <c r="P77" t="s" s="2">
@@ -11423,7 +11420,7 @@
         <v>79</v>
       </c>
       <c r="AF77" t="s" s="2">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="AG77" t="s" s="2">
         <v>90</v>
@@ -11438,27 +11435,27 @@
         <v>102</v>
       </c>
       <c r="AK77" t="s" s="2">
+        <v>400</v>
+      </c>
+      <c r="AL77" t="s" s="2">
         <v>401</v>
       </c>
-      <c r="AL77" t="s" s="2">
+      <c r="AM77" t="s" s="2">
         <v>402</v>
       </c>
-      <c r="AM77" t="s" s="2">
+      <c r="AN77" t="s" s="2">
         <v>403</v>
       </c>
-      <c r="AN77" t="s" s="2">
+      <c r="AO77" t="s" s="2">
         <v>404</v>
-      </c>
-      <c r="AO77" t="s" s="2">
-        <v>405</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s" s="2">
+        <v>409</v>
+      </c>
+      <c r="B78" t="s" s="2">
         <v>410</v>
-      </c>
-      <c r="B78" t="s" s="2">
-        <v>411</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
@@ -11484,10 +11481,10 @@
         <v>151</v>
       </c>
       <c r="L78" t="s" s="2">
+        <v>411</v>
+      </c>
+      <c r="M78" t="s" s="2">
         <v>412</v>
-      </c>
-      <c r="M78" t="s" s="2">
-        <v>413</v>
       </c>
       <c r="N78" s="2"/>
       <c r="O78" s="2"/>
@@ -11570,10 +11567,10 @@
     </row>
     <row r="79">
       <c r="A79" t="s" s="2">
+        <v>413</v>
+      </c>
+      <c r="B79" t="s" s="2">
         <v>414</v>
-      </c>
-      <c r="B79" t="s" s="2">
-        <v>415</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" t="s" s="2">
@@ -11683,13 +11680,13 @@
     </row>
     <row r="80">
       <c r="A80" t="s" s="2">
+        <v>415</v>
+      </c>
+      <c r="B80" t="s" s="2">
+        <v>414</v>
+      </c>
+      <c r="C80" t="s" s="2">
         <v>416</v>
-      </c>
-      <c r="B80" t="s" s="2">
-        <v>415</v>
-      </c>
-      <c r="C80" t="s" s="2">
-        <v>417</v>
       </c>
       <c r="D80" t="s" s="2">
         <v>79</v>
@@ -11711,13 +11708,13 @@
         <v>79</v>
       </c>
       <c r="K80" t="s" s="2">
+        <v>417</v>
+      </c>
+      <c r="L80" t="s" s="2">
         <v>418</v>
       </c>
-      <c r="L80" t="s" s="2">
+      <c r="M80" t="s" s="2">
         <v>419</v>
-      </c>
-      <c r="M80" t="s" s="2">
-        <v>420</v>
       </c>
       <c r="N80" s="2"/>
       <c r="O80" s="2"/>
@@ -11800,10 +11797,10 @@
     </row>
     <row r="81">
       <c r="A81" t="s" s="2">
+        <v>420</v>
+      </c>
+      <c r="B81" t="s" s="2">
         <v>421</v>
-      </c>
-      <c r="B81" t="s" s="2">
-        <v>422</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -11915,10 +11912,10 @@
     </row>
     <row r="82">
       <c r="A82" t="s" s="2">
+        <v>422</v>
+      </c>
+      <c r="B82" t="s" s="2">
         <v>423</v>
-      </c>
-      <c r="B82" t="s" s="2">
-        <v>424</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -12030,10 +12027,10 @@
     </row>
     <row r="83">
       <c r="A83" t="s" s="2">
+        <v>424</v>
+      </c>
+      <c r="B83" t="s" s="2">
         <v>425</v>
-      </c>
-      <c r="B83" t="s" s="2">
-        <v>426</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -12073,7 +12070,7 @@
       </c>
       <c r="Q83" s="2"/>
       <c r="R83" t="s" s="2">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="S83" t="s" s="2">
         <v>79</v>
@@ -12147,10 +12144,10 @@
     </row>
     <row r="84">
       <c r="A84" t="s" s="2">
+        <v>427</v>
+      </c>
+      <c r="B84" t="s" s="2">
         <v>428</v>
-      </c>
-      <c r="B84" t="s" s="2">
-        <v>429</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -12210,7 +12207,7 @@
       </c>
       <c r="Y84" s="2"/>
       <c r="Z84" t="s" s="2">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="AA84" t="s" s="2">
         <v>79</v>
@@ -12260,10 +12257,10 @@
     </row>
     <row r="85">
       <c r="A85" t="s" s="2">
+        <v>430</v>
+      </c>
+      <c r="B85" t="s" s="2">
         <v>431</v>
-      </c>
-      <c r="B85" t="s" s="2">
-        <v>432</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
@@ -12286,13 +12283,13 @@
         <v>79</v>
       </c>
       <c r="K85" t="s" s="2">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="L85" t="s" s="2">
+        <v>432</v>
+      </c>
+      <c r="M85" t="s" s="2">
         <v>433</v>
-      </c>
-      <c r="M85" t="s" s="2">
-        <v>434</v>
       </c>
       <c r="N85" s="2"/>
       <c r="O85" s="2"/>
@@ -12343,7 +12340,7 @@
         <v>79</v>
       </c>
       <c r="AF85" t="s" s="2">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="AG85" t="s" s="2">
         <v>80</v>
@@ -12375,10 +12372,10 @@
     </row>
     <row r="86">
       <c r="A86" t="s" s="2">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -12401,13 +12398,13 @@
         <v>79</v>
       </c>
       <c r="K86" t="s" s="2">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="L86" t="s" s="2">
+        <v>436</v>
+      </c>
+      <c r="M86" t="s" s="2">
         <v>437</v>
-      </c>
-      <c r="M86" t="s" s="2">
-        <v>438</v>
       </c>
       <c r="N86" s="2"/>
       <c r="O86" s="2"/>
@@ -12458,7 +12455,7 @@
         <v>79</v>
       </c>
       <c r="AF86" t="s" s="2">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="AG86" t="s" s="2">
         <v>80</v>
@@ -12479,10 +12476,10 @@
         <v>79</v>
       </c>
       <c r="AM86" t="s" s="2">
+        <v>438</v>
+      </c>
+      <c r="AN86" t="s" s="2">
         <v>439</v>
-      </c>
-      <c r="AN86" t="s" s="2">
-        <v>440</v>
       </c>
       <c r="AO86" t="s" s="2">
         <v>79</v>
@@ -12490,10 +12487,10 @@
     </row>
     <row r="87">
       <c r="A87" t="s" s="2">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -12516,16 +12513,16 @@
         <v>91</v>
       </c>
       <c r="K87" t="s" s="2">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="L87" t="s" s="2">
+        <v>441</v>
+      </c>
+      <c r="M87" t="s" s="2">
         <v>442</v>
       </c>
-      <c r="M87" t="s" s="2">
+      <c r="N87" t="s" s="2">
         <v>443</v>
-      </c>
-      <c r="N87" t="s" s="2">
-        <v>444</v>
       </c>
       <c r="O87" s="2"/>
       <c r="P87" t="s" s="2">
@@ -12575,7 +12572,7 @@
         <v>79</v>
       </c>
       <c r="AF87" t="s" s="2">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="AG87" t="s" s="2">
         <v>80</v>
@@ -12593,13 +12590,13 @@
         <v>79</v>
       </c>
       <c r="AL87" t="s" s="2">
+        <v>444</v>
+      </c>
+      <c r="AM87" t="s" s="2">
         <v>445</v>
       </c>
-      <c r="AM87" t="s" s="2">
+      <c r="AN87" t="s" s="2">
         <v>446</v>
-      </c>
-      <c r="AN87" t="s" s="2">
-        <v>447</v>
       </c>
       <c r="AO87" t="s" s="2">
         <v>79</v>
@@ -12607,10 +12604,10 @@
     </row>
     <row r="88">
       <c r="A88" t="s" s="2">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -12636,13 +12633,13 @@
         <v>195</v>
       </c>
       <c r="L88" t="s" s="2">
+        <v>448</v>
+      </c>
+      <c r="M88" t="s" s="2">
         <v>449</v>
       </c>
-      <c r="M88" t="s" s="2">
+      <c r="N88" t="s" s="2">
         <v>450</v>
-      </c>
-      <c r="N88" t="s" s="2">
-        <v>451</v>
       </c>
       <c r="O88" s="2"/>
       <c r="P88" t="s" s="2">
@@ -12668,10 +12665,10 @@
         <v>79</v>
       </c>
       <c r="X88" t="s" s="2">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="Y88" t="s" s="2">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="Z88" t="s" s="2">
         <v>231</v>
@@ -12692,7 +12689,7 @@
         <v>79</v>
       </c>
       <c r="AF88" t="s" s="2">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="AG88" t="s" s="2">
         <v>80</v>
@@ -12710,13 +12707,13 @@
         <v>79</v>
       </c>
       <c r="AL88" t="s" s="2">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="AM88" t="s" s="2">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="AN88" t="s" s="2">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="AO88" t="s" s="2">
         <v>79</v>
@@ -12724,10 +12721,10 @@
     </row>
     <row r="89">
       <c r="A89" t="s" s="2">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -12750,13 +12747,13 @@
         <v>79</v>
       </c>
       <c r="K89" t="s" s="2">
+        <v>454</v>
+      </c>
+      <c r="L89" t="s" s="2">
         <v>455</v>
       </c>
-      <c r="L89" t="s" s="2">
+      <c r="M89" t="s" s="2">
         <v>456</v>
-      </c>
-      <c r="M89" t="s" s="2">
-        <v>457</v>
       </c>
       <c r="N89" s="2"/>
       <c r="O89" s="2"/>
@@ -12807,7 +12804,7 @@
         <v>79</v>
       </c>
       <c r="AF89" t="s" s="2">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="AG89" t="s" s="2">
         <v>80</v>
@@ -12822,16 +12819,16 @@
         <v>102</v>
       </c>
       <c r="AK89" t="s" s="2">
+        <v>457</v>
+      </c>
+      <c r="AL89" t="s" s="2">
         <v>458</v>
       </c>
-      <c r="AL89" t="s" s="2">
+      <c r="AM89" t="s" s="2">
         <v>459</v>
       </c>
-      <c r="AM89" t="s" s="2">
+      <c r="AN89" t="s" s="2">
         <v>460</v>
-      </c>
-      <c r="AN89" t="s" s="2">
-        <v>461</v>
       </c>
       <c r="AO89" t="s" s="2">
         <v>79</v>
@@ -12839,10 +12836,10 @@
     </row>
     <row r="90">
       <c r="A90" t="s" s="2">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -12865,13 +12862,13 @@
         <v>79</v>
       </c>
       <c r="K90" t="s" s="2">
+        <v>462</v>
+      </c>
+      <c r="L90" t="s" s="2">
         <v>463</v>
       </c>
-      <c r="L90" t="s" s="2">
+      <c r="M90" t="s" s="2">
         <v>464</v>
-      </c>
-      <c r="M90" t="s" s="2">
-        <v>465</v>
       </c>
       <c r="N90" s="2"/>
       <c r="O90" s="2"/>
@@ -12922,7 +12919,7 @@
         <v>79</v>
       </c>
       <c r="AF90" t="s" s="2">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="AG90" t="s" s="2">
         <v>80</v>
@@ -12940,24 +12937,24 @@
         <v>79</v>
       </c>
       <c r="AL90" t="s" s="2">
+        <v>465</v>
+      </c>
+      <c r="AM90" t="s" s="2">
         <v>466</v>
       </c>
-      <c r="AM90" t="s" s="2">
+      <c r="AN90" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AO90" t="s" s="2">
         <v>467</v>
-      </c>
-      <c r="AN90" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AO90" t="s" s="2">
-        <v>468</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s" s="2">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -12983,10 +12980,10 @@
         <v>151</v>
       </c>
       <c r="L91" t="s" s="2">
+        <v>469</v>
+      </c>
+      <c r="M91" t="s" s="2">
         <v>470</v>
-      </c>
-      <c r="M91" t="s" s="2">
-        <v>471</v>
       </c>
       <c r="N91" s="2"/>
       <c r="O91" s="2"/>
@@ -13037,7 +13034,7 @@
         <v>79</v>
       </c>
       <c r="AF91" t="s" s="2">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="AG91" t="s" s="2">
         <v>80</v>
@@ -13055,24 +13052,24 @@
         <v>79</v>
       </c>
       <c r="AL91" t="s" s="2">
+        <v>471</v>
+      </c>
+      <c r="AM91" t="s" s="2">
         <v>472</v>
       </c>
-      <c r="AM91" t="s" s="2">
+      <c r="AN91" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AO91" t="s" s="2">
         <v>473</v>
-      </c>
-      <c r="AN91" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AO91" t="s" s="2">
-        <v>474</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s" s="2">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -13095,13 +13092,13 @@
         <v>79</v>
       </c>
       <c r="K92" t="s" s="2">
+        <v>475</v>
+      </c>
+      <c r="L92" t="s" s="2">
         <v>476</v>
       </c>
-      <c r="L92" t="s" s="2">
+      <c r="M92" t="s" s="2">
         <v>477</v>
-      </c>
-      <c r="M92" t="s" s="2">
-        <v>478</v>
       </c>
       <c r="N92" s="2"/>
       <c r="O92" s="2"/>
@@ -13152,7 +13149,7 @@
         <v>79</v>
       </c>
       <c r="AF92" t="s" s="2">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="AG92" t="s" s="2">
         <v>80</v>
@@ -13170,10 +13167,10 @@
         <v>79</v>
       </c>
       <c r="AL92" t="s" s="2">
+        <v>478</v>
+      </c>
+      <c r="AM92" t="s" s="2">
         <v>479</v>
-      </c>
-      <c r="AM92" t="s" s="2">
-        <v>480</v>
       </c>
       <c r="AN92" t="s" s="2">
         <v>79</v>
@@ -13184,10 +13181,10 @@
     </row>
     <row r="93">
       <c r="A93" t="s" s="2">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -13213,10 +13210,10 @@
         <v>195</v>
       </c>
       <c r="L93" t="s" s="2">
+        <v>481</v>
+      </c>
+      <c r="M93" t="s" s="2">
         <v>482</v>
-      </c>
-      <c r="M93" t="s" s="2">
-        <v>483</v>
       </c>
       <c r="N93" s="2"/>
       <c r="O93" s="2"/>
@@ -13243,11 +13240,11 @@
         <v>79</v>
       </c>
       <c r="X93" t="s" s="2">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="Y93" s="2"/>
       <c r="Z93" t="s" s="2">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="AA93" t="s" s="2">
         <v>79</v>
@@ -13265,7 +13262,7 @@
         <v>79</v>
       </c>
       <c r="AF93" t="s" s="2">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="AG93" t="s" s="2">
         <v>80</v>
@@ -13283,24 +13280,24 @@
         <v>79</v>
       </c>
       <c r="AL93" t="s" s="2">
+        <v>484</v>
+      </c>
+      <c r="AM93" t="s" s="2">
         <v>485</v>
       </c>
-      <c r="AM93" t="s" s="2">
+      <c r="AN93" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AO93" t="s" s="2">
         <v>486</v>
-      </c>
-      <c r="AN93" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AO93" t="s" s="2">
-        <v>487</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="s" s="2">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
@@ -13326,10 +13323,10 @@
         <v>195</v>
       </c>
       <c r="L94" t="s" s="2">
+        <v>488</v>
+      </c>
+      <c r="M94" t="s" s="2">
         <v>489</v>
-      </c>
-      <c r="M94" t="s" s="2">
-        <v>490</v>
       </c>
       <c r="N94" s="2"/>
       <c r="O94" s="2"/>
@@ -13356,11 +13353,11 @@
         <v>79</v>
       </c>
       <c r="X94" t="s" s="2">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="Y94" s="2"/>
       <c r="Z94" t="s" s="2">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="AA94" t="s" s="2">
         <v>79</v>
@@ -13378,7 +13375,7 @@
         <v>79</v>
       </c>
       <c r="AF94" t="s" s="2">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="AG94" t="s" s="2">
         <v>80</v>
@@ -13396,24 +13393,24 @@
         <v>79</v>
       </c>
       <c r="AL94" t="s" s="2">
+        <v>491</v>
+      </c>
+      <c r="AM94" t="s" s="2">
         <v>492</v>
       </c>
-      <c r="AM94" t="s" s="2">
+      <c r="AN94" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AO94" t="s" s="2">
         <v>493</v>
-      </c>
-      <c r="AN94" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AO94" t="s" s="2">
-        <v>494</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="s" s="2">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -13436,13 +13433,13 @@
         <v>79</v>
       </c>
       <c r="K95" t="s" s="2">
+        <v>495</v>
+      </c>
+      <c r="L95" t="s" s="2">
         <v>496</v>
       </c>
-      <c r="L95" t="s" s="2">
+      <c r="M95" t="s" s="2">
         <v>497</v>
-      </c>
-      <c r="M95" t="s" s="2">
-        <v>498</v>
       </c>
       <c r="N95" s="2"/>
       <c r="O95" s="2"/>
@@ -13493,7 +13490,7 @@
         <v>79</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>80</v>
@@ -13511,10 +13508,10 @@
         <v>79</v>
       </c>
       <c r="AL95" t="s" s="2">
+        <v>498</v>
+      </c>
+      <c r="AM95" t="s" s="2">
         <v>499</v>
-      </c>
-      <c r="AM95" t="s" s="2">
-        <v>500</v>
       </c>
       <c r="AN95" t="s" s="2">
         <v>79</v>
@@ -13525,10 +13522,10 @@
     </row>
     <row r="96">
       <c r="A96" t="s" s="2">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -13551,13 +13548,13 @@
         <v>91</v>
       </c>
       <c r="K96" t="s" s="2">
+        <v>501</v>
+      </c>
+      <c r="L96" t="s" s="2">
         <v>502</v>
       </c>
-      <c r="L96" t="s" s="2">
+      <c r="M96" t="s" s="2">
         <v>503</v>
-      </c>
-      <c r="M96" t="s" s="2">
-        <v>504</v>
       </c>
       <c r="N96" s="2"/>
       <c r="O96" s="2"/>
@@ -13596,7 +13593,7 @@
         <v>79</v>
       </c>
       <c r="AB96" t="s" s="2">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="AC96" s="2"/>
       <c r="AD96" t="s" s="2">
@@ -13606,7 +13603,7 @@
         <v>139</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>80</v>
@@ -13621,13 +13618,13 @@
         <v>102</v>
       </c>
       <c r="AK96" t="s" s="2">
+        <v>505</v>
+      </c>
+      <c r="AL96" t="s" s="2">
         <v>506</v>
       </c>
-      <c r="AL96" t="s" s="2">
+      <c r="AM96" t="s" s="2">
         <v>507</v>
-      </c>
-      <c r="AM96" t="s" s="2">
-        <v>508</v>
       </c>
       <c r="AN96" t="s" s="2">
         <v>79</v>
@@ -13638,10 +13635,10 @@
     </row>
     <row r="97">
       <c r="A97" t="s" s="2">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -13753,10 +13750,10 @@
     </row>
     <row r="98">
       <c r="A98" t="s" s="2">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -13870,14 +13867,14 @@
     </row>
     <row r="99">
       <c r="A99" t="s" s="2">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="E99" s="2"/>
       <c r="F99" t="s" s="2">
@@ -13899,10 +13896,10 @@
         <v>135</v>
       </c>
       <c r="L99" t="s" s="2">
+        <v>512</v>
+      </c>
+      <c r="M99" t="s" s="2">
         <v>513</v>
-      </c>
-      <c r="M99" t="s" s="2">
-        <v>514</v>
       </c>
       <c r="N99" t="s" s="2">
         <v>171</v>
@@ -13957,7 +13954,7 @@
         <v>79</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>80</v>
@@ -13989,10 +13986,10 @@
     </row>
     <row r="100">
       <c r="A100" t="s" s="2">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -14018,10 +14015,10 @@
         <v>195</v>
       </c>
       <c r="L100" t="s" s="2">
+        <v>516</v>
+      </c>
+      <c r="M100" t="s" s="2">
         <v>517</v>
-      </c>
-      <c r="M100" t="s" s="2">
-        <v>518</v>
       </c>
       <c r="N100" s="2"/>
       <c r="O100" s="2"/>
@@ -14048,14 +14045,14 @@
         <v>79</v>
       </c>
       <c r="X100" t="s" s="2">
+        <v>518</v>
+      </c>
+      <c r="Y100" t="s" s="2">
         <v>519</v>
       </c>
-      <c r="Y100" t="s" s="2">
+      <c r="Z100" t="s" s="2">
         <v>520</v>
       </c>
-      <c r="Z100" t="s" s="2">
-        <v>521</v>
-      </c>
       <c r="AA100" t="s" s="2">
         <v>79</v>
       </c>
@@ -14072,7 +14069,7 @@
         <v>79</v>
       </c>
       <c r="AF100" t="s" s="2">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="AG100" t="s" s="2">
         <v>80</v>
@@ -14087,13 +14084,13 @@
         <v>102</v>
       </c>
       <c r="AK100" t="s" s="2">
+        <v>521</v>
+      </c>
+      <c r="AL100" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM100" t="s" s="2">
         <v>522</v>
-      </c>
-      <c r="AL100" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM100" t="s" s="2">
-        <v>523</v>
       </c>
       <c r="AN100" t="s" s="2">
         <v>79</v>
@@ -14104,10 +14101,10 @@
     </row>
     <row r="101">
       <c r="A101" t="s" s="2">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -14130,16 +14127,16 @@
         <v>91</v>
       </c>
       <c r="K101" t="s" s="2">
+        <v>524</v>
+      </c>
+      <c r="L101" t="s" s="2">
         <v>525</v>
       </c>
-      <c r="L101" t="s" s="2">
+      <c r="M101" t="s" s="2">
         <v>526</v>
       </c>
-      <c r="M101" t="s" s="2">
+      <c r="N101" t="s" s="2">
         <v>527</v>
-      </c>
-      <c r="N101" t="s" s="2">
-        <v>528</v>
       </c>
       <c r="O101" s="2"/>
       <c r="P101" t="s" s="2">
@@ -14189,7 +14186,7 @@
         <v>79</v>
       </c>
       <c r="AF101" t="s" s="2">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="AG101" t="s" s="2">
         <v>90</v>
@@ -14204,16 +14201,16 @@
         <v>102</v>
       </c>
       <c r="AK101" t="s" s="2">
+        <v>528</v>
+      </c>
+      <c r="AL101" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM101" t="s" s="2">
         <v>529</v>
       </c>
-      <c r="AL101" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM101" t="s" s="2">
+      <c r="AN101" t="s" s="2">
         <v>530</v>
-      </c>
-      <c r="AN101" t="s" s="2">
-        <v>531</v>
       </c>
       <c r="AO101" t="s" s="2">
         <v>79</v>
@@ -14221,13 +14218,13 @@
     </row>
     <row r="102">
       <c r="A102" t="s" s="2">
+        <v>531</v>
+      </c>
+      <c r="B102" t="s" s="2">
+        <v>500</v>
+      </c>
+      <c r="C102" t="s" s="2">
         <v>532</v>
-      </c>
-      <c r="B102" t="s" s="2">
-        <v>501</v>
-      </c>
-      <c r="C102" t="s" s="2">
-        <v>533</v>
       </c>
       <c r="D102" t="s" s="2">
         <v>79</v>
@@ -14249,13 +14246,13 @@
         <v>91</v>
       </c>
       <c r="K102" t="s" s="2">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L102" t="s" s="2">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="M102" t="s" s="2">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="N102" s="2"/>
       <c r="O102" s="2"/>
@@ -14306,7 +14303,7 @@
         <v>79</v>
       </c>
       <c r="AF102" t="s" s="2">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="AG102" t="s" s="2">
         <v>80</v>
@@ -14321,13 +14318,13 @@
         <v>102</v>
       </c>
       <c r="AK102" t="s" s="2">
+        <v>505</v>
+      </c>
+      <c r="AL102" t="s" s="2">
         <v>506</v>
       </c>
-      <c r="AL102" t="s" s="2">
+      <c r="AM102" t="s" s="2">
         <v>507</v>
-      </c>
-      <c r="AM102" t="s" s="2">
-        <v>508</v>
       </c>
       <c r="AN102" t="s" s="2">
         <v>79</v>
@@ -14338,10 +14335,10 @@
     </row>
     <row r="103">
       <c r="A103" t="s" s="2">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B103" t="s" s="2">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" t="s" s="2">
@@ -14453,10 +14450,10 @@
     </row>
     <row r="104">
       <c r="A104" t="s" s="2">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B104" t="s" s="2">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -14570,14 +14567,14 @@
     </row>
     <row r="105">
       <c r="A105" t="s" s="2">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="C105" s="2"/>
       <c r="D105" t="s" s="2">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="E105" s="2"/>
       <c r="F105" t="s" s="2">
@@ -14599,10 +14596,10 @@
         <v>135</v>
       </c>
       <c r="L105" t="s" s="2">
+        <v>512</v>
+      </c>
+      <c r="M105" t="s" s="2">
         <v>513</v>
-      </c>
-      <c r="M105" t="s" s="2">
-        <v>514</v>
       </c>
       <c r="N105" t="s" s="2">
         <v>171</v>
@@ -14657,7 +14654,7 @@
         <v>79</v>
       </c>
       <c r="AF105" t="s" s="2">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="AG105" t="s" s="2">
         <v>80</v>
@@ -14689,10 +14686,10 @@
     </row>
     <row r="106">
       <c r="A106" t="s" s="2">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B106" t="s" s="2">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" t="s" s="2">
@@ -14718,10 +14715,10 @@
         <v>195</v>
       </c>
       <c r="L106" t="s" s="2">
+        <v>516</v>
+      </c>
+      <c r="M106" t="s" s="2">
         <v>517</v>
-      </c>
-      <c r="M106" t="s" s="2">
-        <v>518</v>
       </c>
       <c r="N106" s="2"/>
       <c r="O106" s="2"/>
@@ -14733,7 +14730,7 @@
         <v>79</v>
       </c>
       <c r="S106" t="s" s="2">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="T106" t="s" s="2">
         <v>79</v>
@@ -14748,14 +14745,14 @@
         <v>79</v>
       </c>
       <c r="X106" t="s" s="2">
+        <v>518</v>
+      </c>
+      <c r="Y106" t="s" s="2">
         <v>519</v>
       </c>
-      <c r="Y106" t="s" s="2">
+      <c r="Z106" t="s" s="2">
         <v>520</v>
       </c>
-      <c r="Z106" t="s" s="2">
-        <v>521</v>
-      </c>
       <c r="AA106" t="s" s="2">
         <v>79</v>
       </c>
@@ -14772,7 +14769,7 @@
         <v>79</v>
       </c>
       <c r="AF106" t="s" s="2">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="AG106" t="s" s="2">
         <v>80</v>
@@ -14787,13 +14784,13 @@
         <v>102</v>
       </c>
       <c r="AK106" t="s" s="2">
+        <v>521</v>
+      </c>
+      <c r="AL106" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM106" t="s" s="2">
         <v>522</v>
-      </c>
-      <c r="AL106" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM106" t="s" s="2">
-        <v>523</v>
       </c>
       <c r="AN106" t="s" s="2">
         <v>79</v>
@@ -14804,10 +14801,10 @@
     </row>
     <row r="107">
       <c r="A107" t="s" s="2">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B107" t="s" s="2">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" t="s" s="2">
@@ -14830,16 +14827,16 @@
         <v>91</v>
       </c>
       <c r="K107" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="L107" t="s" s="2">
+        <v>525</v>
+      </c>
+      <c r="M107" t="s" s="2">
         <v>526</v>
       </c>
-      <c r="M107" t="s" s="2">
+      <c r="N107" t="s" s="2">
         <v>527</v>
-      </c>
-      <c r="N107" t="s" s="2">
-        <v>528</v>
       </c>
       <c r="O107" s="2"/>
       <c r="P107" t="s" s="2">
@@ -14889,7 +14886,7 @@
         <v>79</v>
       </c>
       <c r="AF107" t="s" s="2">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="AG107" t="s" s="2">
         <v>90</v>
@@ -14904,16 +14901,16 @@
         <v>102</v>
       </c>
       <c r="AK107" t="s" s="2">
+        <v>528</v>
+      </c>
+      <c r="AL107" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM107" t="s" s="2">
         <v>529</v>
       </c>
-      <c r="AL107" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM107" t="s" s="2">
+      <c r="AN107" t="s" s="2">
         <v>530</v>
-      </c>
-      <c r="AN107" t="s" s="2">
-        <v>531</v>
       </c>
       <c r="AO107" t="s" s="2">
         <v>79</v>
@@ -14921,10 +14918,10 @@
     </row>
     <row r="108">
       <c r="A108" t="s" s="2">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B108" t="s" s="2">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" t="s" s="2">
@@ -14947,13 +14944,13 @@
         <v>91</v>
       </c>
       <c r="K108" t="s" s="2">
+        <v>542</v>
+      </c>
+      <c r="L108" t="s" s="2">
         <v>543</v>
       </c>
-      <c r="L108" t="s" s="2">
+      <c r="M108" t="s" s="2">
         <v>544</v>
-      </c>
-      <c r="M108" t="s" s="2">
-        <v>545</v>
       </c>
       <c r="N108" s="2"/>
       <c r="O108" s="2"/>
@@ -15004,7 +15001,7 @@
         <v>79</v>
       </c>
       <c r="AF108" t="s" s="2">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="AG108" t="s" s="2">
         <v>80</v>
@@ -15019,13 +15016,13 @@
         <v>102</v>
       </c>
       <c r="AK108" t="s" s="2">
+        <v>545</v>
+      </c>
+      <c r="AL108" t="s" s="2">
         <v>546</v>
       </c>
-      <c r="AL108" t="s" s="2">
+      <c r="AM108" t="s" s="2">
         <v>547</v>
-      </c>
-      <c r="AM108" t="s" s="2">
-        <v>548</v>
       </c>
       <c r="AN108" t="s" s="2">
         <v>79</v>
@@ -15036,10 +15033,10 @@
     </row>
     <row r="109">
       <c r="A109" t="s" s="2">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="B109" t="s" s="2">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="C109" s="2"/>
       <c r="D109" t="s" s="2">
@@ -15151,10 +15148,10 @@
     </row>
     <row r="110">
       <c r="A110" t="s" s="2">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B110" t="s" s="2">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C110" s="2"/>
       <c r="D110" t="s" s="2">
@@ -15268,10 +15265,10 @@
     </row>
     <row r="111">
       <c r="A111" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B111" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="C111" s="2"/>
       <c r="D111" t="s" s="2">
@@ -15294,16 +15291,16 @@
         <v>91</v>
       </c>
       <c r="K111" t="s" s="2">
+        <v>551</v>
+      </c>
+      <c r="L111" t="s" s="2">
         <v>552</v>
       </c>
-      <c r="L111" t="s" s="2">
+      <c r="M111" t="s" s="2">
         <v>553</v>
       </c>
-      <c r="M111" t="s" s="2">
+      <c r="N111" t="s" s="2">
         <v>554</v>
-      </c>
-      <c r="N111" t="s" s="2">
-        <v>555</v>
       </c>
       <c r="O111" s="2"/>
       <c r="P111" t="s" s="2">
@@ -15353,7 +15350,7 @@
         <v>79</v>
       </c>
       <c r="AF111" t="s" s="2">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="AG111" t="s" s="2">
         <v>80</v>
@@ -15374,7 +15371,7 @@
         <v>133</v>
       </c>
       <c r="AM111" t="s" s="2">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="AN111" t="s" s="2">
         <v>79</v>
@@ -15385,10 +15382,10 @@
     </row>
     <row r="112">
       <c r="A112" t="s" s="2">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B112" t="s" s="2">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" t="s" s="2">
@@ -15411,13 +15408,13 @@
         <v>91</v>
       </c>
       <c r="K112" t="s" s="2">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="L112" t="s" s="2">
+        <v>558</v>
+      </c>
+      <c r="M112" t="s" s="2">
         <v>559</v>
-      </c>
-      <c r="M112" t="s" s="2">
-        <v>560</v>
       </c>
       <c r="N112" s="2"/>
       <c r="O112" s="2"/>
@@ -15468,7 +15465,7 @@
         <v>79</v>
       </c>
       <c r="AF112" t="s" s="2">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="AG112" t="s" s="2">
         <v>80</v>
@@ -15489,7 +15486,7 @@
         <v>133</v>
       </c>
       <c r="AM112" t="s" s="2">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="AN112" t="s" s="2">
         <v>79</v>
@@ -15500,10 +15497,10 @@
     </row>
     <row r="113">
       <c r="A113" t="s" s="2">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="B113" t="s" s="2">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="C113" s="2"/>
       <c r="D113" t="s" s="2">
@@ -15526,13 +15523,13 @@
         <v>91</v>
       </c>
       <c r="K113" t="s" s="2">
+        <v>563</v>
+      </c>
+      <c r="L113" t="s" s="2">
         <v>564</v>
       </c>
-      <c r="L113" t="s" s="2">
+      <c r="M113" t="s" s="2">
         <v>565</v>
-      </c>
-      <c r="M113" t="s" s="2">
-        <v>566</v>
       </c>
       <c r="N113" s="2"/>
       <c r="O113" s="2"/>
@@ -15583,7 +15580,7 @@
         <v>79</v>
       </c>
       <c r="AF113" t="s" s="2">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="AG113" t="s" s="2">
         <v>90</v>
@@ -15604,7 +15601,7 @@
         <v>133</v>
       </c>
       <c r="AM113" t="s" s="2">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="AN113" t="s" s="2">
         <v>79</v>
@@ -15615,10 +15612,10 @@
     </row>
     <row r="114">
       <c r="A114" t="s" s="2">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B114" t="s" s="2">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="C114" s="2"/>
       <c r="D114" t="s" s="2">
@@ -15644,10 +15641,10 @@
         <v>195</v>
       </c>
       <c r="L114" t="s" s="2">
+        <v>569</v>
+      </c>
+      <c r="M114" t="s" s="2">
         <v>570</v>
-      </c>
-      <c r="M114" t="s" s="2">
-        <v>571</v>
       </c>
       <c r="N114" s="2"/>
       <c r="O114" s="2"/>
@@ -15674,14 +15671,14 @@
         <v>79</v>
       </c>
       <c r="X114" t="s" s="2">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="Y114" t="s" s="2">
+        <v>571</v>
+      </c>
+      <c r="Z114" t="s" s="2">
         <v>572</v>
       </c>
-      <c r="Z114" t="s" s="2">
-        <v>573</v>
-      </c>
       <c r="AA114" t="s" s="2">
         <v>79</v>
       </c>
@@ -15698,7 +15695,7 @@
         <v>79</v>
       </c>
       <c r="AF114" t="s" s="2">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="AG114" t="s" s="2">
         <v>80</v>
@@ -15713,13 +15710,13 @@
         <v>102</v>
       </c>
       <c r="AK114" t="s" s="2">
+        <v>573</v>
+      </c>
+      <c r="AL114" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM114" t="s" s="2">
         <v>574</v>
-      </c>
-      <c r="AL114" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM114" t="s" s="2">
-        <v>575</v>
       </c>
       <c r="AN114" t="s" s="2">
         <v>79</v>
@@ -15730,10 +15727,10 @@
     </row>
     <row r="115">
       <c r="A115" t="s" s="2">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="B115" t="s" s="2">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="C115" s="2"/>
       <c r="D115" t="s" s="2">
@@ -15756,13 +15753,13 @@
         <v>79</v>
       </c>
       <c r="K115" t="s" s="2">
+        <v>576</v>
+      </c>
+      <c r="L115" t="s" s="2">
         <v>577</v>
       </c>
-      <c r="L115" t="s" s="2">
+      <c r="M115" t="s" s="2">
         <v>578</v>
-      </c>
-      <c r="M115" t="s" s="2">
-        <v>579</v>
       </c>
       <c r="N115" s="2"/>
       <c r="O115" s="2"/>
@@ -15813,7 +15810,7 @@
         <v>79</v>
       </c>
       <c r="AF115" t="s" s="2">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="AG115" t="s" s="2">
         <v>80</v>
@@ -15828,7 +15825,7 @@
         <v>102</v>
       </c>
       <c r="AK115" t="s" s="2">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AL115" t="s" s="2">
         <v>79</v>
@@ -15845,10 +15842,10 @@
     </row>
     <row r="116">
       <c r="A116" t="s" s="2">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="B116" t="s" s="2">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C116" s="2"/>
       <c r="D116" t="s" s="2">
@@ -15871,23 +15868,23 @@
         <v>91</v>
       </c>
       <c r="K116" t="s" s="2">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="L116" t="s" s="2">
+        <v>581</v>
+      </c>
+      <c r="M116" t="s" s="2">
         <v>582</v>
       </c>
-      <c r="M116" t="s" s="2">
+      <c r="N116" t="s" s="2">
         <v>583</v>
-      </c>
-      <c r="N116" t="s" s="2">
-        <v>584</v>
       </c>
       <c r="O116" s="2"/>
       <c r="P116" t="s" s="2">
         <v>79</v>
       </c>
       <c r="Q116" t="s" s="2">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="R116" t="s" s="2">
         <v>79</v>
@@ -15932,7 +15929,7 @@
         <v>79</v>
       </c>
       <c r="AF116" t="s" s="2">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="AG116" t="s" s="2">
         <v>80</v>
@@ -15950,7 +15947,7 @@
         <v>79</v>
       </c>
       <c r="AL116" t="s" s="2">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="AM116" t="s" s="2">
         <v>133</v>
@@ -15964,10 +15961,10 @@
     </row>
     <row r="117">
       <c r="A117" t="s" s="2">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B117" t="s" s="2">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="C117" s="2"/>
       <c r="D117" t="s" s="2">
@@ -15993,10 +15990,10 @@
         <v>195</v>
       </c>
       <c r="L117" t="s" s="2">
+        <v>587</v>
+      </c>
+      <c r="M117" t="s" s="2">
         <v>588</v>
-      </c>
-      <c r="M117" t="s" s="2">
-        <v>589</v>
       </c>
       <c r="N117" s="2"/>
       <c r="O117" s="2"/>
@@ -16023,14 +16020,14 @@
         <v>79</v>
       </c>
       <c r="X117" t="s" s="2">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="Y117" t="s" s="2">
+        <v>589</v>
+      </c>
+      <c r="Z117" t="s" s="2">
         <v>590</v>
       </c>
-      <c r="Z117" t="s" s="2">
-        <v>591</v>
-      </c>
       <c r="AA117" t="s" s="2">
         <v>79</v>
       </c>
@@ -16047,7 +16044,7 @@
         <v>79</v>
       </c>
       <c r="AF117" t="s" s="2">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AG117" t="s" s="2">
         <v>80</v>
@@ -16079,10 +16076,10 @@
     </row>
     <row r="118">
       <c r="A118" t="s" s="2">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B118" t="s" s="2">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C118" s="2"/>
       <c r="D118" t="s" s="2">
@@ -16105,13 +16102,13 @@
         <v>79</v>
       </c>
       <c r="K118" t="s" s="2">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L118" t="s" s="2">
+        <v>592</v>
+      </c>
+      <c r="M118" t="s" s="2">
         <v>593</v>
-      </c>
-      <c r="M118" t="s" s="2">
-        <v>594</v>
       </c>
       <c r="N118" s="2"/>
       <c r="O118" s="2"/>
@@ -16162,7 +16159,7 @@
         <v>79</v>
       </c>
       <c r="AF118" t="s" s="2">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="AG118" t="s" s="2">
         <v>80</v>
@@ -16174,7 +16171,7 @@
         <v>79</v>
       </c>
       <c r="AJ118" t="s" s="2">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="AK118" t="s" s="2">
         <v>79</v>
@@ -16194,10 +16191,10 @@
     </row>
     <row r="119">
       <c r="A119" t="s" s="2">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B119" t="s" s="2">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="C119" s="2"/>
       <c r="D119" t="s" s="2">
@@ -16309,10 +16306,10 @@
     </row>
     <row r="120">
       <c r="A120" t="s" s="2">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B120" t="s" s="2">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="C120" s="2"/>
       <c r="D120" t="s" s="2">
@@ -16426,14 +16423,14 @@
     </row>
     <row r="121">
       <c r="A121" t="s" s="2">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B121" t="s" s="2">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="C121" s="2"/>
       <c r="D121" t="s" s="2">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="E121" s="2"/>
       <c r="F121" t="s" s="2">
@@ -16455,10 +16452,10 @@
         <v>135</v>
       </c>
       <c r="L121" t="s" s="2">
+        <v>512</v>
+      </c>
+      <c r="M121" t="s" s="2">
         <v>513</v>
-      </c>
-      <c r="M121" t="s" s="2">
-        <v>514</v>
       </c>
       <c r="N121" t="s" s="2">
         <v>171</v>
@@ -16513,7 +16510,7 @@
         <v>79</v>
       </c>
       <c r="AF121" t="s" s="2">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="AG121" t="s" s="2">
         <v>80</v>
@@ -16545,10 +16542,10 @@
     </row>
     <row r="122">
       <c r="A122" t="s" s="2">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B122" t="s" s="2">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="C122" s="2"/>
       <c r="D122" t="s" s="2">
@@ -16574,10 +16571,10 @@
         <v>151</v>
       </c>
       <c r="L122" t="s" s="2">
+        <v>599</v>
+      </c>
+      <c r="M122" t="s" s="2">
         <v>600</v>
-      </c>
-      <c r="M122" t="s" s="2">
-        <v>601</v>
       </c>
       <c r="N122" s="2"/>
       <c r="O122" s="2"/>
@@ -16628,7 +16625,7 @@
         <v>79</v>
       </c>
       <c r="AF122" t="s" s="2">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="AG122" t="s" s="2">
         <v>80</v>
@@ -16646,7 +16643,7 @@
         <v>79</v>
       </c>
       <c r="AL122" t="s" s="2">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="AM122" t="s" s="2">
         <v>133</v>
@@ -16660,10 +16657,10 @@
     </row>
     <row r="123">
       <c r="A123" t="s" s="2">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B123" t="s" s="2">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="C123" s="2"/>
       <c r="D123" t="s" s="2">
@@ -16689,10 +16686,10 @@
         <v>104</v>
       </c>
       <c r="L123" t="s" s="2">
+        <v>603</v>
+      </c>
+      <c r="M123" t="s" s="2">
         <v>604</v>
-      </c>
-      <c r="M123" t="s" s="2">
-        <v>605</v>
       </c>
       <c r="N123" s="2"/>
       <c r="O123" s="2"/>
@@ -16743,7 +16740,7 @@
         <v>79</v>
       </c>
       <c r="AF123" t="s" s="2">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="AG123" t="s" s="2">
         <v>80</v>
@@ -16775,10 +16772,10 @@
     </row>
     <row r="124">
       <c r="A124" t="s" s="2">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B124" t="s" s="2">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C124" s="2"/>
       <c r="D124" t="s" s="2">
@@ -16801,13 +16798,13 @@
         <v>79</v>
       </c>
       <c r="K124" t="s" s="2">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="L124" t="s" s="2">
+        <v>606</v>
+      </c>
+      <c r="M124" t="s" s="2">
         <v>607</v>
-      </c>
-      <c r="M124" t="s" s="2">
-        <v>608</v>
       </c>
       <c r="N124" s="2"/>
       <c r="O124" s="2"/>
@@ -16858,7 +16855,7 @@
         <v>79</v>
       </c>
       <c r="AF124" t="s" s="2">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="AG124" t="s" s="2">
         <v>80</v>
@@ -16876,7 +16873,7 @@
         <v>79</v>
       </c>
       <c r="AL124" t="s" s="2">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="AM124" t="s" s="2">
         <v>133</v>
@@ -16890,10 +16887,10 @@
     </row>
     <row r="125">
       <c r="A125" t="s" s="2">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B125" t="s" s="2">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="C125" s="2"/>
       <c r="D125" t="s" s="2">
@@ -16916,13 +16913,13 @@
         <v>79</v>
       </c>
       <c r="K125" t="s" s="2">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="L125" t="s" s="2">
+        <v>610</v>
+      </c>
+      <c r="M125" t="s" s="2">
         <v>611</v>
-      </c>
-      <c r="M125" t="s" s="2">
-        <v>612</v>
       </c>
       <c r="N125" s="2"/>
       <c r="O125" s="2"/>
@@ -16973,7 +16970,7 @@
         <v>79</v>
       </c>
       <c r="AF125" t="s" s="2">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="AG125" t="s" s="2">
         <v>80</v>
@@ -16991,7 +16988,7 @@
         <v>79</v>
       </c>
       <c r="AL125" t="s" s="2">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="AM125" t="s" s="2">
         <v>133</v>
@@ -17005,10 +17002,10 @@
     </row>
     <row r="126">
       <c r="A126" t="s" s="2">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B126" t="s" s="2">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="C126" s="2"/>
       <c r="D126" t="s" s="2">
@@ -17034,10 +17031,10 @@
         <v>195</v>
       </c>
       <c r="L126" t="s" s="2">
+        <v>614</v>
+      </c>
+      <c r="M126" t="s" s="2">
         <v>615</v>
-      </c>
-      <c r="M126" t="s" s="2">
-        <v>616</v>
       </c>
       <c r="N126" s="2"/>
       <c r="O126" s="2"/>
@@ -17064,14 +17061,14 @@
         <v>79</v>
       </c>
       <c r="X126" t="s" s="2">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="Y126" t="s" s="2">
+        <v>616</v>
+      </c>
+      <c r="Z126" t="s" s="2">
         <v>617</v>
       </c>
-      <c r="Z126" t="s" s="2">
-        <v>618</v>
-      </c>
       <c r="AA126" t="s" s="2">
         <v>79</v>
       </c>
@@ -17088,7 +17085,7 @@
         <v>79</v>
       </c>
       <c r="AF126" t="s" s="2">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="AG126" t="s" s="2">
         <v>80</v>
@@ -17106,7 +17103,7 @@
         <v>79</v>
       </c>
       <c r="AL126" t="s" s="2">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="AM126" t="s" s="2">
         <v>133</v>
@@ -17120,10 +17117,10 @@
     </row>
     <row r="127">
       <c r="A127" t="s" s="2">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B127" t="s" s="2">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="C127" s="2"/>
       <c r="D127" t="s" s="2">
@@ -17149,10 +17146,10 @@
         <v>195</v>
       </c>
       <c r="L127" t="s" s="2">
+        <v>620</v>
+      </c>
+      <c r="M127" t="s" s="2">
         <v>621</v>
-      </c>
-      <c r="M127" t="s" s="2">
-        <v>622</v>
       </c>
       <c r="N127" s="2"/>
       <c r="O127" s="2"/>
@@ -17179,14 +17176,14 @@
         <v>79</v>
       </c>
       <c r="X127" t="s" s="2">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="Y127" t="s" s="2">
+        <v>622</v>
+      </c>
+      <c r="Z127" t="s" s="2">
         <v>623</v>
       </c>
-      <c r="Z127" t="s" s="2">
-        <v>624</v>
-      </c>
       <c r="AA127" t="s" s="2">
         <v>79</v>
       </c>
@@ -17203,7 +17200,7 @@
         <v>79</v>
       </c>
       <c r="AF127" t="s" s="2">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="AG127" t="s" s="2">
         <v>80</v>
@@ -17235,10 +17232,10 @@
     </row>
     <row r="128">
       <c r="A128" t="s" s="2">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B128" t="s" s="2">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="C128" s="2"/>
       <c r="D128" t="s" s="2">
@@ -17261,16 +17258,16 @@
         <v>79</v>
       </c>
       <c r="K128" t="s" s="2">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L128" t="s" s="2">
+        <v>625</v>
+      </c>
+      <c r="M128" t="s" s="2">
         <v>626</v>
       </c>
-      <c r="M128" t="s" s="2">
+      <c r="N128" t="s" s="2">
         <v>627</v>
-      </c>
-      <c r="N128" t="s" s="2">
-        <v>628</v>
       </c>
       <c r="O128" s="2"/>
       <c r="P128" t="s" s="2">
@@ -17320,7 +17317,7 @@
         <v>79</v>
       </c>
       <c r="AF128" t="s" s="2">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="AG128" t="s" s="2">
         <v>80</v>
@@ -17338,10 +17335,10 @@
         <v>79</v>
       </c>
       <c r="AL128" t="s" s="2">
+        <v>628</v>
+      </c>
+      <c r="AM128" t="s" s="2">
         <v>629</v>
-      </c>
-      <c r="AM128" t="s" s="2">
-        <v>630</v>
       </c>
       <c r="AN128" t="s" s="2">
         <v>79</v>
@@ -17352,10 +17349,10 @@
     </row>
     <row r="129">
       <c r="A129" t="s" s="2">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B129" t="s" s="2">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="C129" s="2"/>
       <c r="D129" t="s" s="2">
@@ -17467,10 +17464,10 @@
     </row>
     <row r="130">
       <c r="A130" t="s" s="2">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B130" t="s" s="2">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="C130" s="2"/>
       <c r="D130" t="s" s="2">
@@ -17584,14 +17581,14 @@
     </row>
     <row r="131">
       <c r="A131" t="s" s="2">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B131" t="s" s="2">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="C131" s="2"/>
       <c r="D131" t="s" s="2">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="E131" s="2"/>
       <c r="F131" t="s" s="2">
@@ -17613,10 +17610,10 @@
         <v>135</v>
       </c>
       <c r="L131" t="s" s="2">
+        <v>512</v>
+      </c>
+      <c r="M131" t="s" s="2">
         <v>513</v>
-      </c>
-      <c r="M131" t="s" s="2">
-        <v>514</v>
       </c>
       <c r="N131" t="s" s="2">
         <v>171</v>
@@ -17671,7 +17668,7 @@
         <v>79</v>
       </c>
       <c r="AF131" t="s" s="2">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="AG131" t="s" s="2">
         <v>80</v>
@@ -17703,10 +17700,10 @@
     </row>
     <row r="132">
       <c r="A132" t="s" s="2">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B132" t="s" s="2">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="C132" s="2"/>
       <c r="D132" t="s" s="2">
@@ -17729,13 +17726,13 @@
         <v>79</v>
       </c>
       <c r="K132" t="s" s="2">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="L132" t="s" s="2">
+        <v>634</v>
+      </c>
+      <c r="M132" t="s" s="2">
         <v>635</v>
-      </c>
-      <c r="M132" t="s" s="2">
-        <v>636</v>
       </c>
       <c r="N132" s="2"/>
       <c r="O132" s="2"/>
@@ -17786,7 +17783,7 @@
         <v>79</v>
       </c>
       <c r="AF132" t="s" s="2">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="AG132" t="s" s="2">
         <v>80</v>
@@ -17804,10 +17801,10 @@
         <v>79</v>
       </c>
       <c r="AL132" t="s" s="2">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="AM132" t="s" s="2">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="AN132" t="s" s="2">
         <v>79</v>
@@ -17818,10 +17815,10 @@
     </row>
     <row r="133">
       <c r="A133" t="s" s="2">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="B133" t="s" s="2">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="C133" s="2"/>
       <c r="D133" t="s" s="2">
@@ -17844,13 +17841,13 @@
         <v>79</v>
       </c>
       <c r="K133" t="s" s="2">
+        <v>638</v>
+      </c>
+      <c r="L133" t="s" s="2">
         <v>639</v>
       </c>
-      <c r="L133" t="s" s="2">
+      <c r="M133" t="s" s="2">
         <v>640</v>
-      </c>
-      <c r="M133" t="s" s="2">
-        <v>641</v>
       </c>
       <c r="N133" s="2"/>
       <c r="O133" s="2"/>
@@ -17901,7 +17898,7 @@
         <v>79</v>
       </c>
       <c r="AF133" t="s" s="2">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="AG133" t="s" s="2">
         <v>80</v>
@@ -17919,10 +17916,10 @@
         <v>79</v>
       </c>
       <c r="AL133" t="s" s="2">
+        <v>641</v>
+      </c>
+      <c r="AM133" t="s" s="2">
         <v>642</v>
-      </c>
-      <c r="AM133" t="s" s="2">
-        <v>643</v>
       </c>
       <c r="AN133" t="s" s="2">
         <v>79</v>
@@ -17933,10 +17930,10 @@
     </row>
     <row r="134">
       <c r="A134" t="s" s="2">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B134" t="s" s="2">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="C134" s="2"/>
       <c r="D134" t="s" s="2">
@@ -17959,13 +17956,13 @@
         <v>79</v>
       </c>
       <c r="K134" t="s" s="2">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="L134" t="s" s="2">
+        <v>644</v>
+      </c>
+      <c r="M134" t="s" s="2">
         <v>645</v>
-      </c>
-      <c r="M134" t="s" s="2">
-        <v>646</v>
       </c>
       <c r="N134" s="2"/>
       <c r="O134" s="2"/>
@@ -18016,7 +18013,7 @@
         <v>79</v>
       </c>
       <c r="AF134" t="s" s="2">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="AG134" t="s" s="2">
         <v>80</v>
@@ -18034,10 +18031,10 @@
         <v>79</v>
       </c>
       <c r="AL134" t="s" s="2">
+        <v>646</v>
+      </c>
+      <c r="AM134" t="s" s="2">
         <v>647</v>
-      </c>
-      <c r="AM134" t="s" s="2">
-        <v>648</v>
       </c>
       <c r="AN134" t="s" s="2">
         <v>79</v>
@@ -18048,10 +18045,10 @@
     </row>
     <row r="135">
       <c r="A135" t="s" s="2">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B135" t="s" s="2">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="C135" s="2"/>
       <c r="D135" t="s" s="2">
@@ -18074,13 +18071,13 @@
         <v>79</v>
       </c>
       <c r="K135" t="s" s="2">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L135" t="s" s="2">
+        <v>649</v>
+      </c>
+      <c r="M135" t="s" s="2">
         <v>650</v>
-      </c>
-      <c r="M135" t="s" s="2">
-        <v>651</v>
       </c>
       <c r="N135" s="2"/>
       <c r="O135" s="2"/>
@@ -18131,7 +18128,7 @@
         <v>79</v>
       </c>
       <c r="AF135" t="s" s="2">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="AG135" t="s" s="2">
         <v>80</v>
@@ -18163,10 +18160,10 @@
     </row>
     <row r="136">
       <c r="A136" t="s" s="2">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="B136" t="s" s="2">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="C136" s="2"/>
       <c r="D136" t="s" s="2">
@@ -18278,10 +18275,10 @@
     </row>
     <row r="137">
       <c r="A137" t="s" s="2">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B137" t="s" s="2">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="C137" s="2"/>
       <c r="D137" t="s" s="2">
@@ -18395,14 +18392,14 @@
     </row>
     <row r="138">
       <c r="A138" t="s" s="2">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="B138" t="s" s="2">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="C138" s="2"/>
       <c r="D138" t="s" s="2">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="E138" s="2"/>
       <c r="F138" t="s" s="2">
@@ -18424,10 +18421,10 @@
         <v>135</v>
       </c>
       <c r="L138" t="s" s="2">
+        <v>512</v>
+      </c>
+      <c r="M138" t="s" s="2">
         <v>513</v>
-      </c>
-      <c r="M138" t="s" s="2">
-        <v>514</v>
       </c>
       <c r="N138" t="s" s="2">
         <v>171</v>
@@ -18482,7 +18479,7 @@
         <v>79</v>
       </c>
       <c r="AF138" t="s" s="2">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="AG138" t="s" s="2">
         <v>80</v>
@@ -18514,10 +18511,10 @@
     </row>
     <row r="139">
       <c r="A139" t="s" s="2">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B139" t="s" s="2">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="C139" s="2"/>
       <c r="D139" t="s" s="2">
@@ -18543,10 +18540,10 @@
         <v>151</v>
       </c>
       <c r="L139" t="s" s="2">
+        <v>655</v>
+      </c>
+      <c r="M139" t="s" s="2">
         <v>656</v>
-      </c>
-      <c r="M139" t="s" s="2">
-        <v>657</v>
       </c>
       <c r="N139" s="2"/>
       <c r="O139" s="2"/>
@@ -18573,11 +18570,11 @@
         <v>79</v>
       </c>
       <c r="X139" t="s" s="2">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="Y139" s="2"/>
       <c r="Z139" t="s" s="2">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="AA139" t="s" s="2">
         <v>79</v>
@@ -18595,7 +18592,7 @@
         <v>79</v>
       </c>
       <c r="AF139" t="s" s="2">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="AG139" t="s" s="2">
         <v>80</v>
@@ -18627,10 +18624,10 @@
     </row>
     <row r="140">
       <c r="A140" t="s" s="2">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B140" t="s" s="2">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="C140" s="2"/>
       <c r="D140" t="s" s="2">
@@ -18653,13 +18650,13 @@
         <v>79</v>
       </c>
       <c r="K140" t="s" s="2">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L140" t="s" s="2">
+        <v>659</v>
+      </c>
+      <c r="M140" t="s" s="2">
         <v>660</v>
-      </c>
-      <c r="M140" t="s" s="2">
-        <v>661</v>
       </c>
       <c r="N140" s="2"/>
       <c r="O140" s="2"/>
@@ -18710,7 +18707,7 @@
         <v>79</v>
       </c>
       <c r="AF140" t="s" s="2">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="AG140" t="s" s="2">
         <v>80</v>
@@ -18742,10 +18739,10 @@
     </row>
     <row r="141">
       <c r="A141" t="s" s="2">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B141" t="s" s="2">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C141" s="2"/>
       <c r="D141" t="s" s="2">
@@ -18771,10 +18768,10 @@
         <v>195</v>
       </c>
       <c r="L141" t="s" s="2">
+        <v>662</v>
+      </c>
+      <c r="M141" t="s" s="2">
         <v>663</v>
-      </c>
-      <c r="M141" t="s" s="2">
-        <v>664</v>
       </c>
       <c r="N141" s="2"/>
       <c r="O141" s="2"/>
@@ -18804,11 +18801,11 @@
         <v>114</v>
       </c>
       <c r="Y141" t="s" s="2">
+        <v>664</v>
+      </c>
+      <c r="Z141" t="s" s="2">
         <v>665</v>
       </c>
-      <c r="Z141" t="s" s="2">
-        <v>666</v>
-      </c>
       <c r="AA141" t="s" s="2">
         <v>79</v>
       </c>
@@ -18825,7 +18822,7 @@
         <v>79</v>
       </c>
       <c r="AF141" t="s" s="2">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="AG141" t="s" s="2">
         <v>80</v>
@@ -18857,10 +18854,10 @@
     </row>
     <row r="142">
       <c r="A142" t="s" s="2">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B142" t="s" s="2">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="C142" s="2"/>
       <c r="D142" t="s" s="2">
@@ -18883,16 +18880,16 @@
         <v>79</v>
       </c>
       <c r="K142" t="s" s="2">
+        <v>667</v>
+      </c>
+      <c r="L142" t="s" s="2">
         <v>668</v>
       </c>
-      <c r="L142" t="s" s="2">
+      <c r="M142" t="s" s="2">
         <v>669</v>
       </c>
-      <c r="M142" t="s" s="2">
+      <c r="N142" t="s" s="2">
         <v>670</v>
-      </c>
-      <c r="N142" t="s" s="2">
-        <v>671</v>
       </c>
       <c r="O142" s="2"/>
       <c r="P142" t="s" s="2">
@@ -18930,7 +18927,7 @@
         <v>79</v>
       </c>
       <c r="AB142" t="s" s="2">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="AC142" s="2"/>
       <c r="AD142" t="s" s="2">
@@ -18940,7 +18937,7 @@
         <v>139</v>
       </c>
       <c r="AF142" t="s" s="2">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="AG142" t="s" s="2">
         <v>90</v>
@@ -18972,13 +18969,13 @@
     </row>
     <row r="143">
       <c r="A143" t="s" s="2">
+        <v>671</v>
+      </c>
+      <c r="B143" t="s" s="2">
+        <v>666</v>
+      </c>
+      <c r="C143" t="s" s="2">
         <v>672</v>
-      </c>
-      <c r="B143" t="s" s="2">
-        <v>667</v>
-      </c>
-      <c r="C143" t="s" s="2">
-        <v>673</v>
       </c>
       <c r="D143" t="s" s="2">
         <v>79</v>
@@ -19000,16 +18997,16 @@
         <v>79</v>
       </c>
       <c r="K143" t="s" s="2">
+        <v>673</v>
+      </c>
+      <c r="L143" t="s" s="2">
         <v>674</v>
       </c>
-      <c r="L143" t="s" s="2">
-        <v>675</v>
-      </c>
       <c r="M143" t="s" s="2">
+        <v>669</v>
+      </c>
+      <c r="N143" t="s" s="2">
         <v>670</v>
-      </c>
-      <c r="N143" t="s" s="2">
-        <v>671</v>
       </c>
       <c r="O143" s="2"/>
       <c r="P143" t="s" s="2">
@@ -19059,7 +19056,7 @@
         <v>79</v>
       </c>
       <c r="AF143" t="s" s="2">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="AG143" t="s" s="2">
         <v>90</v>
@@ -19091,10 +19088,10 @@
     </row>
     <row r="144">
       <c r="A144" t="s" s="2">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="B144" t="s" s="2">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="C144" s="2"/>
       <c r="D144" t="s" s="2">
@@ -19117,16 +19114,16 @@
         <v>79</v>
       </c>
       <c r="K144" t="s" s="2">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="L144" t="s" s="2">
+        <v>676</v>
+      </c>
+      <c r="M144" t="s" s="2">
         <v>677</v>
       </c>
-      <c r="M144" t="s" s="2">
-        <v>678</v>
-      </c>
       <c r="N144" t="s" s="2">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="O144" s="2"/>
       <c r="P144" t="s" s="2">
@@ -19176,7 +19173,7 @@
         <v>79</v>
       </c>
       <c r="AF144" t="s" s="2">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="AG144" t="s" s="2">
         <v>80</v>

</xml_diff>

<commit_message>
refactor: suppression identifier ^short (non contraint dans FRCore)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com> 60d2deb4f4f6d0a50e2085425b8464890e3cb2c9
</commit_message>
<xml_diff>
--- a/nr-doc-core-immunization/ig/StructureDefinition-fr-core-immunization.xlsx
+++ b/nr-doc-core-immunization/ig/StructureDefinition-fr-core-immunization.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-22T13:13:25+00:00</t>
+    <t>2026-06-22T13:33:44+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -854,7 +854,7 @@
 </t>
   </si>
   <si>
-    <t>Identifiant</t>
+    <t>Identifier of the immunization</t>
   </si>
   <si>
     <t>A unique identifier assigned to this immunization record.</t>

</xml_diff>

<commit_message>
feat: ajout ^short protocolApplied.series avec codes autorisés
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com> d358a82cda133ea0cd908474715b715147d24096
</commit_message>
<xml_diff>
--- a/nr-doc-core-immunization/ig/StructureDefinition-fr-core-immunization.xlsx
+++ b/nr-doc-core-immunization/ig/StructureDefinition-fr-core-immunization.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-22T13:33:44+00:00</t>
+    <t>2026-06-22T13:44:32+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2044,7 +2044,7 @@
     <t>Immunization.protocolApplied.series</t>
   </si>
   <si>
-    <t>Name of vaccine series</t>
+    <t>Type de vaccination : BOOSTER (Rappel de vaccin) | IMMUNIZ (Vaccination sans autre précision) | INITIMMUNIZ (1ère série vaccinante)</t>
   </si>
   <si>
     <t>One possible path to achieve presumed immunity against a disease - within the context of an authority.</t>

</xml_diff>

<commit_message>
refactor: suppression référence obsolète à FRMedicationAdministrationDocument dans la description
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com> 35b3c96f818a9998fdc65c496cbba62dd6ad3238
</commit_message>
<xml_diff>
--- a/nr-doc-core-immunization/ig/StructureDefinition-fr-core-immunization.xlsx
+++ b/nr-doc-core-immunization/ig/StructureDefinition-fr-core-immunization.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-22T14:24:08+00:00</t>
+    <t>2026-06-22T14:26:05+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -85,8 +85,7 @@
   </si>
   <si>
     <t>FRCoreImmunizationProfile permet de décrire l'administration d'un vaccin.
- - Il permet également de décrire pourquoi un vaccin n'a pas été réalisé.
- - Ce profil hérite de la structuration, des contraintes et des vocabulaires définis dans le profil FRMedicationAdministrationDocument sauf mentions précisées ci-après.</t>
+ - Il permet également de décrire pourquoi un vaccin n'a pas été réalisé.</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>

<commit_message>
fix: aligne immunization avec PR #177 Doc Core
- Suppression de la référence à data-absent-reason sur occurrence[x]
- Mise à jour du bloc commenté performer/auteur : extension racine
  au lieu de performer.actor.extension
- Ajout alias $v2-0443

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com> c3ffd48d41228624bb0ee6b572dd3e1bb071381c
</commit_message>
<xml_diff>
--- a/nr-doc-core-immunization/ig/StructureDefinition-fr-core-immunization.xlsx
+++ b/nr-doc-core-immunization/ig/StructureDefinition-fr-core-immunization.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4975" uniqueCount="623">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4975" uniqueCount="622">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-29T10:25:23+00:00</t>
+    <t>2026-06-29T15:19:05+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1072,7 +1072,7 @@
     <t>Date de la vaccination</t>
   </si>
   <si>
-    <t>Si la date de la vaccination est inconnue, utiliser l'extension data-absent-reason précisant pourquoi elle n'est pas connue.</t>
+    <t>Date vaccine administered or was to be administered.</t>
   </si>
   <si>
     <t>When immunizations are given a specific date and time should always be known.   When immunizations are patient reported, a specific date might not be known.  Although partial dates are allowed, an adult patient might not be able to recall the year a childhood immunization was given. An exact date is always preferable, but the use of the String data type is acceptable when an exact date is not known. A small number of vaccines (e.g. live oral typhoid vaccine) are given as a series of patient self-administered dose over a span of time. In cases like this, often, only the first dose (typically a provider supervised dose) is recorded with the occurrence indicating the date/time of the first dose.</t>
@@ -1107,9 +1107,6 @@
   </si>
   <si>
     <t>Vaccine administration date</t>
-  </si>
-  <si>
-    <t>Date vaccine administered or was to be administered.</t>
   </si>
   <si>
     <t>Immunization.occurrence[x]:occurrenceDateTime.id</t>
@@ -10140,7 +10137,7 @@
         <v>351</v>
       </c>
       <c r="M68" t="s" s="2">
-        <v>352</v>
+        <v>340</v>
       </c>
       <c r="N68" t="s" s="2">
         <v>341</v>
@@ -10225,10 +10222,10 @@
     </row>
     <row r="69">
       <c r="A69" t="s" s="2">
+        <v>352</v>
+      </c>
+      <c r="B69" t="s" s="2">
         <v>353</v>
-      </c>
-      <c r="B69" t="s" s="2">
-        <v>354</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -10254,10 +10251,10 @@
         <v>151</v>
       </c>
       <c r="L69" t="s" s="2">
+        <v>354</v>
+      </c>
+      <c r="M69" t="s" s="2">
         <v>355</v>
-      </c>
-      <c r="M69" t="s" s="2">
-        <v>356</v>
       </c>
       <c r="N69" s="2"/>
       <c r="O69" s="2"/>
@@ -10340,10 +10337,10 @@
     </row>
     <row r="70">
       <c r="A70" t="s" s="2">
+        <v>356</v>
+      </c>
+      <c r="B70" t="s" s="2">
         <v>357</v>
-      </c>
-      <c r="B70" t="s" s="2">
-        <v>358</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -10453,13 +10450,13 @@
     </row>
     <row r="71">
       <c r="A71" t="s" s="2">
+        <v>358</v>
+      </c>
+      <c r="B71" t="s" s="2">
+        <v>357</v>
+      </c>
+      <c r="C71" t="s" s="2">
         <v>359</v>
-      </c>
-      <c r="B71" t="s" s="2">
-        <v>358</v>
-      </c>
-      <c r="C71" t="s" s="2">
-        <v>360</v>
       </c>
       <c r="D71" t="s" s="2">
         <v>79</v>
@@ -10481,13 +10478,13 @@
         <v>79</v>
       </c>
       <c r="K71" t="s" s="2">
+        <v>360</v>
+      </c>
+      <c r="L71" t="s" s="2">
         <v>361</v>
       </c>
-      <c r="L71" t="s" s="2">
+      <c r="M71" t="s" s="2">
         <v>362</v>
-      </c>
-      <c r="M71" t="s" s="2">
-        <v>363</v>
       </c>
       <c r="N71" s="2"/>
       <c r="O71" s="2"/>
@@ -10570,10 +10567,10 @@
     </row>
     <row r="72">
       <c r="A72" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="B72" t="s" s="2">
         <v>364</v>
-      </c>
-      <c r="B72" t="s" s="2">
-        <v>365</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -10685,10 +10682,10 @@
     </row>
     <row r="73">
       <c r="A73" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="B73" t="s" s="2">
         <v>366</v>
-      </c>
-      <c r="B73" t="s" s="2">
-        <v>367</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -10800,10 +10797,10 @@
     </row>
     <row r="74">
       <c r="A74" t="s" s="2">
+        <v>367</v>
+      </c>
+      <c r="B74" t="s" s="2">
         <v>368</v>
-      </c>
-      <c r="B74" t="s" s="2">
-        <v>369</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
@@ -10843,7 +10840,7 @@
       </c>
       <c r="Q74" s="2"/>
       <c r="R74" t="s" s="2">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="S74" t="s" s="2">
         <v>79</v>
@@ -10917,10 +10914,10 @@
     </row>
     <row r="75">
       <c r="A75" t="s" s="2">
+        <v>370</v>
+      </c>
+      <c r="B75" t="s" s="2">
         <v>371</v>
-      </c>
-      <c r="B75" t="s" s="2">
-        <v>372</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
@@ -10980,7 +10977,7 @@
       </c>
       <c r="Y75" s="2"/>
       <c r="Z75" t="s" s="2">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="AA75" t="s" s="2">
         <v>79</v>
@@ -11030,10 +11027,10 @@
     </row>
     <row r="76">
       <c r="A76" t="s" s="2">
+        <v>373</v>
+      </c>
+      <c r="B76" t="s" s="2">
         <v>374</v>
-      </c>
-      <c r="B76" t="s" s="2">
-        <v>375</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -11059,10 +11056,10 @@
         <v>338</v>
       </c>
       <c r="L76" t="s" s="2">
+        <v>375</v>
+      </c>
+      <c r="M76" t="s" s="2">
         <v>376</v>
-      </c>
-      <c r="M76" t="s" s="2">
-        <v>377</v>
       </c>
       <c r="N76" s="2"/>
       <c r="O76" s="2"/>
@@ -11113,7 +11110,7 @@
         <v>79</v>
       </c>
       <c r="AF76" t="s" s="2">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="AG76" t="s" s="2">
         <v>80</v>
@@ -11145,10 +11142,10 @@
     </row>
     <row r="77">
       <c r="A77" t="s" s="2">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -11174,10 +11171,10 @@
         <v>338</v>
       </c>
       <c r="L77" t="s" s="2">
+        <v>379</v>
+      </c>
+      <c r="M77" t="s" s="2">
         <v>380</v>
-      </c>
-      <c r="M77" t="s" s="2">
-        <v>381</v>
       </c>
       <c r="N77" s="2"/>
       <c r="O77" s="2"/>
@@ -11228,7 +11225,7 @@
         <v>79</v>
       </c>
       <c r="AF77" t="s" s="2">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="AG77" t="s" s="2">
         <v>80</v>
@@ -11249,10 +11246,10 @@
         <v>79</v>
       </c>
       <c r="AM77" t="s" s="2">
+        <v>381</v>
+      </c>
+      <c r="AN77" t="s" s="2">
         <v>382</v>
-      </c>
-      <c r="AN77" t="s" s="2">
-        <v>383</v>
       </c>
       <c r="AO77" t="s" s="2">
         <v>79</v>
@@ -11260,10 +11257,10 @@
     </row>
     <row r="78">
       <c r="A78" t="s" s="2">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
@@ -11286,16 +11283,16 @@
         <v>91</v>
       </c>
       <c r="K78" t="s" s="2">
+        <v>384</v>
+      </c>
+      <c r="L78" t="s" s="2">
         <v>385</v>
       </c>
-      <c r="L78" t="s" s="2">
+      <c r="M78" t="s" s="2">
         <v>386</v>
       </c>
-      <c r="M78" t="s" s="2">
+      <c r="N78" t="s" s="2">
         <v>387</v>
-      </c>
-      <c r="N78" t="s" s="2">
-        <v>388</v>
       </c>
       <c r="O78" s="2"/>
       <c r="P78" t="s" s="2">
@@ -11345,7 +11342,7 @@
         <v>79</v>
       </c>
       <c r="AF78" t="s" s="2">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="AG78" t="s" s="2">
         <v>80</v>
@@ -11363,13 +11360,13 @@
         <v>79</v>
       </c>
       <c r="AL78" t="s" s="2">
+        <v>388</v>
+      </c>
+      <c r="AM78" t="s" s="2">
         <v>389</v>
       </c>
-      <c r="AM78" t="s" s="2">
+      <c r="AN78" t="s" s="2">
         <v>390</v>
-      </c>
-      <c r="AN78" t="s" s="2">
-        <v>391</v>
       </c>
       <c r="AO78" t="s" s="2">
         <v>79</v>
@@ -11377,10 +11374,10 @@
     </row>
     <row r="79">
       <c r="A79" t="s" s="2">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" t="s" s="2">
@@ -11406,13 +11403,13 @@
         <v>195</v>
       </c>
       <c r="L79" t="s" s="2">
+        <v>392</v>
+      </c>
+      <c r="M79" t="s" s="2">
         <v>393</v>
       </c>
-      <c r="M79" t="s" s="2">
+      <c r="N79" t="s" s="2">
         <v>394</v>
-      </c>
-      <c r="N79" t="s" s="2">
-        <v>395</v>
       </c>
       <c r="O79" s="2"/>
       <c r="P79" t="s" s="2">
@@ -11441,7 +11438,7 @@
         <v>283</v>
       </c>
       <c r="Y79" t="s" s="2">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="Z79" t="s" s="2">
         <v>231</v>
@@ -11462,7 +11459,7 @@
         <v>79</v>
       </c>
       <c r="AF79" t="s" s="2">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="AG79" t="s" s="2">
         <v>80</v>
@@ -11480,13 +11477,13 @@
         <v>79</v>
       </c>
       <c r="AL79" t="s" s="2">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="AM79" t="s" s="2">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="AN79" t="s" s="2">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="AO79" t="s" s="2">
         <v>79</v>
@@ -11494,10 +11491,10 @@
     </row>
     <row r="80">
       <c r="A80" t="s" s="2">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" t="s" s="2">
@@ -11520,13 +11517,13 @@
         <v>79</v>
       </c>
       <c r="K80" t="s" s="2">
+        <v>398</v>
+      </c>
+      <c r="L80" t="s" s="2">
         <v>399</v>
       </c>
-      <c r="L80" t="s" s="2">
+      <c r="M80" t="s" s="2">
         <v>400</v>
-      </c>
-      <c r="M80" t="s" s="2">
-        <v>401</v>
       </c>
       <c r="N80" s="2"/>
       <c r="O80" s="2"/>
@@ -11577,7 +11574,7 @@
         <v>79</v>
       </c>
       <c r="AF80" t="s" s="2">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="AG80" t="s" s="2">
         <v>80</v>
@@ -11592,16 +11589,16 @@
         <v>102</v>
       </c>
       <c r="AK80" t="s" s="2">
+        <v>401</v>
+      </c>
+      <c r="AL80" t="s" s="2">
         <v>402</v>
       </c>
-      <c r="AL80" t="s" s="2">
+      <c r="AM80" t="s" s="2">
         <v>403</v>
       </c>
-      <c r="AM80" t="s" s="2">
+      <c r="AN80" t="s" s="2">
         <v>404</v>
-      </c>
-      <c r="AN80" t="s" s="2">
-        <v>405</v>
       </c>
       <c r="AO80" t="s" s="2">
         <v>79</v>
@@ -11609,10 +11606,10 @@
     </row>
     <row r="81">
       <c r="A81" t="s" s="2">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -11635,13 +11632,13 @@
         <v>79</v>
       </c>
       <c r="K81" t="s" s="2">
+        <v>406</v>
+      </c>
+      <c r="L81" t="s" s="2">
         <v>407</v>
       </c>
-      <c r="L81" t="s" s="2">
+      <c r="M81" t="s" s="2">
         <v>408</v>
-      </c>
-      <c r="M81" t="s" s="2">
-        <v>409</v>
       </c>
       <c r="N81" s="2"/>
       <c r="O81" s="2"/>
@@ -11692,7 +11689,7 @@
         <v>79</v>
       </c>
       <c r="AF81" t="s" s="2">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="AG81" t="s" s="2">
         <v>80</v>
@@ -11710,24 +11707,24 @@
         <v>79</v>
       </c>
       <c r="AL81" t="s" s="2">
+        <v>409</v>
+      </c>
+      <c r="AM81" t="s" s="2">
         <v>410</v>
       </c>
-      <c r="AM81" t="s" s="2">
+      <c r="AN81" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AO81" t="s" s="2">
         <v>411</v>
-      </c>
-      <c r="AN81" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AO81" t="s" s="2">
-        <v>412</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s" s="2">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -11753,10 +11750,10 @@
         <v>151</v>
       </c>
       <c r="L82" t="s" s="2">
+        <v>413</v>
+      </c>
+      <c r="M82" t="s" s="2">
         <v>414</v>
-      </c>
-      <c r="M82" t="s" s="2">
-        <v>415</v>
       </c>
       <c r="N82" s="2"/>
       <c r="O82" s="2"/>
@@ -11807,7 +11804,7 @@
         <v>79</v>
       </c>
       <c r="AF82" t="s" s="2">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="AG82" t="s" s="2">
         <v>80</v>
@@ -11825,24 +11822,24 @@
         <v>79</v>
       </c>
       <c r="AL82" t="s" s="2">
+        <v>415</v>
+      </c>
+      <c r="AM82" t="s" s="2">
         <v>416</v>
       </c>
-      <c r="AM82" t="s" s="2">
+      <c r="AN82" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AO82" t="s" s="2">
         <v>417</v>
-      </c>
-      <c r="AN82" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AO82" t="s" s="2">
-        <v>418</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="s" s="2">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -11865,13 +11862,13 @@
         <v>79</v>
       </c>
       <c r="K83" t="s" s="2">
+        <v>419</v>
+      </c>
+      <c r="L83" t="s" s="2">
         <v>420</v>
       </c>
-      <c r="L83" t="s" s="2">
+      <c r="M83" t="s" s="2">
         <v>421</v>
-      </c>
-      <c r="M83" t="s" s="2">
-        <v>422</v>
       </c>
       <c r="N83" s="2"/>
       <c r="O83" s="2"/>
@@ -11922,7 +11919,7 @@
         <v>79</v>
       </c>
       <c r="AF83" t="s" s="2">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>80</v>
@@ -11940,10 +11937,10 @@
         <v>79</v>
       </c>
       <c r="AL83" t="s" s="2">
+        <v>422</v>
+      </c>
+      <c r="AM83" t="s" s="2">
         <v>423</v>
-      </c>
-      <c r="AM83" t="s" s="2">
-        <v>424</v>
       </c>
       <c r="AN83" t="s" s="2">
         <v>79</v>
@@ -11954,10 +11951,10 @@
     </row>
     <row r="84">
       <c r="A84" t="s" s="2">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B84" t="s" s="2">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -11983,10 +11980,10 @@
         <v>195</v>
       </c>
       <c r="L84" t="s" s="2">
+        <v>425</v>
+      </c>
+      <c r="M84" t="s" s="2">
         <v>426</v>
-      </c>
-      <c r="M84" t="s" s="2">
-        <v>427</v>
       </c>
       <c r="N84" s="2"/>
       <c r="O84" s="2"/>
@@ -12017,7 +12014,7 @@
       </c>
       <c r="Y84" s="2"/>
       <c r="Z84" t="s" s="2">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="AA84" t="s" s="2">
         <v>79</v>
@@ -12035,7 +12032,7 @@
         <v>79</v>
       </c>
       <c r="AF84" t="s" s="2">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="AG84" t="s" s="2">
         <v>80</v>
@@ -12053,24 +12050,24 @@
         <v>79</v>
       </c>
       <c r="AL84" t="s" s="2">
+        <v>428</v>
+      </c>
+      <c r="AM84" t="s" s="2">
         <v>429</v>
       </c>
-      <c r="AM84" t="s" s="2">
+      <c r="AN84" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AO84" t="s" s="2">
         <v>430</v>
-      </c>
-      <c r="AN84" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AO84" t="s" s="2">
-        <v>431</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="s" s="2">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
@@ -12096,10 +12093,10 @@
         <v>195</v>
       </c>
       <c r="L85" t="s" s="2">
+        <v>432</v>
+      </c>
+      <c r="M85" t="s" s="2">
         <v>433</v>
-      </c>
-      <c r="M85" t="s" s="2">
-        <v>434</v>
       </c>
       <c r="N85" s="2"/>
       <c r="O85" s="2"/>
@@ -12130,7 +12127,7 @@
       </c>
       <c r="Y85" s="2"/>
       <c r="Z85" t="s" s="2">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="AA85" t="s" s="2">
         <v>79</v>
@@ -12148,7 +12145,7 @@
         <v>79</v>
       </c>
       <c r="AF85" t="s" s="2">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="AG85" t="s" s="2">
         <v>80</v>
@@ -12166,24 +12163,24 @@
         <v>79</v>
       </c>
       <c r="AL85" t="s" s="2">
+        <v>435</v>
+      </c>
+      <c r="AM85" t="s" s="2">
         <v>436</v>
       </c>
-      <c r="AM85" t="s" s="2">
+      <c r="AN85" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AO85" t="s" s="2">
         <v>437</v>
-      </c>
-      <c r="AN85" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AO85" t="s" s="2">
-        <v>438</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s" s="2">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -12206,13 +12203,13 @@
         <v>79</v>
       </c>
       <c r="K86" t="s" s="2">
+        <v>439</v>
+      </c>
+      <c r="L86" t="s" s="2">
         <v>440</v>
       </c>
-      <c r="L86" t="s" s="2">
+      <c r="M86" t="s" s="2">
         <v>441</v>
-      </c>
-      <c r="M86" t="s" s="2">
-        <v>442</v>
       </c>
       <c r="N86" s="2"/>
       <c r="O86" s="2"/>
@@ -12263,7 +12260,7 @@
         <v>79</v>
       </c>
       <c r="AF86" t="s" s="2">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="AG86" t="s" s="2">
         <v>80</v>
@@ -12281,10 +12278,10 @@
         <v>79</v>
       </c>
       <c r="AL86" t="s" s="2">
+        <v>442</v>
+      </c>
+      <c r="AM86" t="s" s="2">
         <v>443</v>
-      </c>
-      <c r="AM86" t="s" s="2">
-        <v>444</v>
       </c>
       <c r="AN86" t="s" s="2">
         <v>79</v>
@@ -12295,10 +12292,10 @@
     </row>
     <row r="87">
       <c r="A87" t="s" s="2">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -12321,13 +12318,13 @@
         <v>91</v>
       </c>
       <c r="K87" t="s" s="2">
+        <v>445</v>
+      </c>
+      <c r="L87" t="s" s="2">
         <v>446</v>
       </c>
-      <c r="L87" t="s" s="2">
+      <c r="M87" t="s" s="2">
         <v>447</v>
-      </c>
-      <c r="M87" t="s" s="2">
-        <v>448</v>
       </c>
       <c r="N87" s="2"/>
       <c r="O87" s="2"/>
@@ -12366,7 +12363,7 @@
         <v>79</v>
       </c>
       <c r="AB87" t="s" s="2">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="AC87" s="2"/>
       <c r="AD87" t="s" s="2">
@@ -12376,7 +12373,7 @@
         <v>139</v>
       </c>
       <c r="AF87" t="s" s="2">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="AG87" t="s" s="2">
         <v>80</v>
@@ -12391,13 +12388,13 @@
         <v>102</v>
       </c>
       <c r="AK87" t="s" s="2">
+        <v>449</v>
+      </c>
+      <c r="AL87" t="s" s="2">
         <v>450</v>
       </c>
-      <c r="AL87" t="s" s="2">
+      <c r="AM87" t="s" s="2">
         <v>451</v>
-      </c>
-      <c r="AM87" t="s" s="2">
-        <v>452</v>
       </c>
       <c r="AN87" t="s" s="2">
         <v>79</v>
@@ -12408,10 +12405,10 @@
     </row>
     <row r="88">
       <c r="A88" t="s" s="2">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -12523,10 +12520,10 @@
     </row>
     <row r="89">
       <c r="A89" t="s" s="2">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -12640,14 +12637,14 @@
     </row>
     <row r="90">
       <c r="A90" t="s" s="2">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="E90" s="2"/>
       <c r="F90" t="s" s="2">
@@ -12669,10 +12666,10 @@
         <v>135</v>
       </c>
       <c r="L90" t="s" s="2">
+        <v>456</v>
+      </c>
+      <c r="M90" t="s" s="2">
         <v>457</v>
-      </c>
-      <c r="M90" t="s" s="2">
-        <v>458</v>
       </c>
       <c r="N90" t="s" s="2">
         <v>171</v>
@@ -12727,7 +12724,7 @@
         <v>79</v>
       </c>
       <c r="AF90" t="s" s="2">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="AG90" t="s" s="2">
         <v>80</v>
@@ -12759,10 +12756,10 @@
     </row>
     <row r="91">
       <c r="A91" t="s" s="2">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -12788,10 +12785,10 @@
         <v>195</v>
       </c>
       <c r="L91" t="s" s="2">
+        <v>460</v>
+      </c>
+      <c r="M91" t="s" s="2">
         <v>461</v>
-      </c>
-      <c r="M91" t="s" s="2">
-        <v>462</v>
       </c>
       <c r="N91" s="2"/>
       <c r="O91" s="2"/>
@@ -12818,14 +12815,14 @@
         <v>79</v>
       </c>
       <c r="X91" t="s" s="2">
+        <v>462</v>
+      </c>
+      <c r="Y91" t="s" s="2">
         <v>463</v>
       </c>
-      <c r="Y91" t="s" s="2">
+      <c r="Z91" t="s" s="2">
         <v>464</v>
       </c>
-      <c r="Z91" t="s" s="2">
-        <v>465</v>
-      </c>
       <c r="AA91" t="s" s="2">
         <v>79</v>
       </c>
@@ -12842,7 +12839,7 @@
         <v>79</v>
       </c>
       <c r="AF91" t="s" s="2">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="AG91" t="s" s="2">
         <v>80</v>
@@ -12857,13 +12854,13 @@
         <v>102</v>
       </c>
       <c r="AK91" t="s" s="2">
+        <v>465</v>
+      </c>
+      <c r="AL91" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM91" t="s" s="2">
         <v>466</v>
-      </c>
-      <c r="AL91" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM91" t="s" s="2">
-        <v>467</v>
       </c>
       <c r="AN91" t="s" s="2">
         <v>79</v>
@@ -12874,10 +12871,10 @@
     </row>
     <row r="92">
       <c r="A92" t="s" s="2">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -12900,16 +12897,16 @@
         <v>91</v>
       </c>
       <c r="K92" t="s" s="2">
+        <v>468</v>
+      </c>
+      <c r="L92" t="s" s="2">
         <v>469</v>
       </c>
-      <c r="L92" t="s" s="2">
+      <c r="M92" t="s" s="2">
         <v>470</v>
       </c>
-      <c r="M92" t="s" s="2">
+      <c r="N92" t="s" s="2">
         <v>471</v>
-      </c>
-      <c r="N92" t="s" s="2">
-        <v>472</v>
       </c>
       <c r="O92" s="2"/>
       <c r="P92" t="s" s="2">
@@ -12959,7 +12956,7 @@
         <v>79</v>
       </c>
       <c r="AF92" t="s" s="2">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="AG92" t="s" s="2">
         <v>90</v>
@@ -12974,16 +12971,16 @@
         <v>102</v>
       </c>
       <c r="AK92" t="s" s="2">
+        <v>472</v>
+      </c>
+      <c r="AL92" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM92" t="s" s="2">
         <v>473</v>
       </c>
-      <c r="AL92" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM92" t="s" s="2">
+      <c r="AN92" t="s" s="2">
         <v>474</v>
-      </c>
-      <c r="AN92" t="s" s="2">
-        <v>475</v>
       </c>
       <c r="AO92" t="s" s="2">
         <v>79</v>
@@ -12991,13 +12988,13 @@
     </row>
     <row r="93">
       <c r="A93" t="s" s="2">
+        <v>475</v>
+      </c>
+      <c r="B93" t="s" s="2">
+        <v>444</v>
+      </c>
+      <c r="C93" t="s" s="2">
         <v>476</v>
-      </c>
-      <c r="B93" t="s" s="2">
-        <v>445</v>
-      </c>
-      <c r="C93" t="s" s="2">
-        <v>477</v>
       </c>
       <c r="D93" t="s" s="2">
         <v>79</v>
@@ -13019,13 +13016,13 @@
         <v>91</v>
       </c>
       <c r="K93" t="s" s="2">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="L93" t="s" s="2">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="M93" t="s" s="2">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="N93" s="2"/>
       <c r="O93" s="2"/>
@@ -13076,7 +13073,7 @@
         <v>79</v>
       </c>
       <c r="AF93" t="s" s="2">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="AG93" t="s" s="2">
         <v>80</v>
@@ -13091,13 +13088,13 @@
         <v>102</v>
       </c>
       <c r="AK93" t="s" s="2">
+        <v>449</v>
+      </c>
+      <c r="AL93" t="s" s="2">
         <v>450</v>
       </c>
-      <c r="AL93" t="s" s="2">
+      <c r="AM93" t="s" s="2">
         <v>451</v>
-      </c>
-      <c r="AM93" t="s" s="2">
-        <v>452</v>
       </c>
       <c r="AN93" t="s" s="2">
         <v>79</v>
@@ -13108,10 +13105,10 @@
     </row>
     <row r="94">
       <c r="A94" t="s" s="2">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
@@ -13223,10 +13220,10 @@
     </row>
     <row r="95">
       <c r="A95" t="s" s="2">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -13340,14 +13337,14 @@
     </row>
     <row r="96">
       <c r="A96" t="s" s="2">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="E96" s="2"/>
       <c r="F96" t="s" s="2">
@@ -13369,10 +13366,10 @@
         <v>135</v>
       </c>
       <c r="L96" t="s" s="2">
+        <v>456</v>
+      </c>
+      <c r="M96" t="s" s="2">
         <v>457</v>
-      </c>
-      <c r="M96" t="s" s="2">
-        <v>458</v>
       </c>
       <c r="N96" t="s" s="2">
         <v>171</v>
@@ -13427,7 +13424,7 @@
         <v>79</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>80</v>
@@ -13459,10 +13456,10 @@
     </row>
     <row r="97">
       <c r="A97" t="s" s="2">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -13488,10 +13485,10 @@
         <v>195</v>
       </c>
       <c r="L97" t="s" s="2">
+        <v>460</v>
+      </c>
+      <c r="M97" t="s" s="2">
         <v>461</v>
-      </c>
-      <c r="M97" t="s" s="2">
-        <v>462</v>
       </c>
       <c r="N97" s="2"/>
       <c r="O97" s="2"/>
@@ -13503,7 +13500,7 @@
         <v>79</v>
       </c>
       <c r="S97" t="s" s="2">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="T97" t="s" s="2">
         <v>79</v>
@@ -13518,14 +13515,14 @@
         <v>79</v>
       </c>
       <c r="X97" t="s" s="2">
+        <v>462</v>
+      </c>
+      <c r="Y97" t="s" s="2">
         <v>463</v>
       </c>
-      <c r="Y97" t="s" s="2">
+      <c r="Z97" t="s" s="2">
         <v>464</v>
       </c>
-      <c r="Z97" t="s" s="2">
-        <v>465</v>
-      </c>
       <c r="AA97" t="s" s="2">
         <v>79</v>
       </c>
@@ -13542,7 +13539,7 @@
         <v>79</v>
       </c>
       <c r="AF97" t="s" s="2">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="AG97" t="s" s="2">
         <v>80</v>
@@ -13557,13 +13554,13 @@
         <v>102</v>
       </c>
       <c r="AK97" t="s" s="2">
+        <v>465</v>
+      </c>
+      <c r="AL97" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM97" t="s" s="2">
         <v>466</v>
-      </c>
-      <c r="AL97" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM97" t="s" s="2">
-        <v>467</v>
       </c>
       <c r="AN97" t="s" s="2">
         <v>79</v>
@@ -13574,10 +13571,10 @@
     </row>
     <row r="98">
       <c r="A98" t="s" s="2">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -13600,16 +13597,16 @@
         <v>91</v>
       </c>
       <c r="K98" t="s" s="2">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="L98" t="s" s="2">
+        <v>469</v>
+      </c>
+      <c r="M98" t="s" s="2">
         <v>470</v>
       </c>
-      <c r="M98" t="s" s="2">
+      <c r="N98" t="s" s="2">
         <v>471</v>
-      </c>
-      <c r="N98" t="s" s="2">
-        <v>472</v>
       </c>
       <c r="O98" s="2"/>
       <c r="P98" t="s" s="2">
@@ -13659,7 +13656,7 @@
         <v>79</v>
       </c>
       <c r="AF98" t="s" s="2">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="AG98" t="s" s="2">
         <v>90</v>
@@ -13674,16 +13671,16 @@
         <v>102</v>
       </c>
       <c r="AK98" t="s" s="2">
+        <v>472</v>
+      </c>
+      <c r="AL98" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM98" t="s" s="2">
         <v>473</v>
       </c>
-      <c r="AL98" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM98" t="s" s="2">
+      <c r="AN98" t="s" s="2">
         <v>474</v>
-      </c>
-      <c r="AN98" t="s" s="2">
-        <v>475</v>
       </c>
       <c r="AO98" t="s" s="2">
         <v>79</v>
@@ -13691,10 +13688,10 @@
     </row>
     <row r="99">
       <c r="A99" t="s" s="2">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
@@ -13717,13 +13714,13 @@
         <v>91</v>
       </c>
       <c r="K99" t="s" s="2">
+        <v>486</v>
+      </c>
+      <c r="L99" t="s" s="2">
         <v>487</v>
       </c>
-      <c r="L99" t="s" s="2">
+      <c r="M99" t="s" s="2">
         <v>488</v>
-      </c>
-      <c r="M99" t="s" s="2">
-        <v>489</v>
       </c>
       <c r="N99" s="2"/>
       <c r="O99" s="2"/>
@@ -13774,7 +13771,7 @@
         <v>79</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>80</v>
@@ -13789,13 +13786,13 @@
         <v>102</v>
       </c>
       <c r="AK99" t="s" s="2">
+        <v>489</v>
+      </c>
+      <c r="AL99" t="s" s="2">
         <v>490</v>
       </c>
-      <c r="AL99" t="s" s="2">
+      <c r="AM99" t="s" s="2">
         <v>491</v>
-      </c>
-      <c r="AM99" t="s" s="2">
-        <v>492</v>
       </c>
       <c r="AN99" t="s" s="2">
         <v>79</v>
@@ -13806,10 +13803,10 @@
     </row>
     <row r="100">
       <c r="A100" t="s" s="2">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -13921,10 +13918,10 @@
     </row>
     <row r="101">
       <c r="A101" t="s" s="2">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -14038,10 +14035,10 @@
     </row>
     <row r="102">
       <c r="A102" t="s" s="2">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -14064,16 +14061,16 @@
         <v>91</v>
       </c>
       <c r="K102" t="s" s="2">
+        <v>495</v>
+      </c>
+      <c r="L102" t="s" s="2">
         <v>496</v>
       </c>
-      <c r="L102" t="s" s="2">
+      <c r="M102" t="s" s="2">
         <v>497</v>
       </c>
-      <c r="M102" t="s" s="2">
+      <c r="N102" t="s" s="2">
         <v>498</v>
-      </c>
-      <c r="N102" t="s" s="2">
-        <v>499</v>
       </c>
       <c r="O102" s="2"/>
       <c r="P102" t="s" s="2">
@@ -14123,7 +14120,7 @@
         <v>79</v>
       </c>
       <c r="AF102" t="s" s="2">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="AG102" t="s" s="2">
         <v>80</v>
@@ -14144,7 +14141,7 @@
         <v>133</v>
       </c>
       <c r="AM102" t="s" s="2">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="AN102" t="s" s="2">
         <v>79</v>
@@ -14155,10 +14152,10 @@
     </row>
     <row r="103">
       <c r="A103" t="s" s="2">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B103" t="s" s="2">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" t="s" s="2">
@@ -14184,10 +14181,10 @@
         <v>338</v>
       </c>
       <c r="L103" t="s" s="2">
+        <v>502</v>
+      </c>
+      <c r="M103" t="s" s="2">
         <v>503</v>
-      </c>
-      <c r="M103" t="s" s="2">
-        <v>504</v>
       </c>
       <c r="N103" s="2"/>
       <c r="O103" s="2"/>
@@ -14238,7 +14235,7 @@
         <v>79</v>
       </c>
       <c r="AF103" t="s" s="2">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="AG103" t="s" s="2">
         <v>80</v>
@@ -14259,7 +14256,7 @@
         <v>133</v>
       </c>
       <c r="AM103" t="s" s="2">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="AN103" t="s" s="2">
         <v>79</v>
@@ -14270,10 +14267,10 @@
     </row>
     <row r="104">
       <c r="A104" t="s" s="2">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="B104" t="s" s="2">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -14296,13 +14293,13 @@
         <v>91</v>
       </c>
       <c r="K104" t="s" s="2">
+        <v>507</v>
+      </c>
+      <c r="L104" t="s" s="2">
         <v>508</v>
       </c>
-      <c r="L104" t="s" s="2">
+      <c r="M104" t="s" s="2">
         <v>509</v>
-      </c>
-      <c r="M104" t="s" s="2">
-        <v>510</v>
       </c>
       <c r="N104" s="2"/>
       <c r="O104" s="2"/>
@@ -14353,7 +14350,7 @@
         <v>79</v>
       </c>
       <c r="AF104" t="s" s="2">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="AG104" t="s" s="2">
         <v>90</v>
@@ -14374,7 +14371,7 @@
         <v>133</v>
       </c>
       <c r="AM104" t="s" s="2">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="AN104" t="s" s="2">
         <v>79</v>
@@ -14385,10 +14382,10 @@
     </row>
     <row r="105">
       <c r="A105" t="s" s="2">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C105" s="2"/>
       <c r="D105" t="s" s="2">
@@ -14414,10 +14411,10 @@
         <v>195</v>
       </c>
       <c r="L105" t="s" s="2">
+        <v>513</v>
+      </c>
+      <c r="M105" t="s" s="2">
         <v>514</v>
-      </c>
-      <c r="M105" t="s" s="2">
-        <v>515</v>
       </c>
       <c r="N105" s="2"/>
       <c r="O105" s="2"/>
@@ -14447,11 +14444,11 @@
         <v>283</v>
       </c>
       <c r="Y105" t="s" s="2">
+        <v>515</v>
+      </c>
+      <c r="Z105" t="s" s="2">
         <v>516</v>
       </c>
-      <c r="Z105" t="s" s="2">
-        <v>517</v>
-      </c>
       <c r="AA105" t="s" s="2">
         <v>79</v>
       </c>
@@ -14468,7 +14465,7 @@
         <v>79</v>
       </c>
       <c r="AF105" t="s" s="2">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="AG105" t="s" s="2">
         <v>80</v>
@@ -14483,13 +14480,13 @@
         <v>102</v>
       </c>
       <c r="AK105" t="s" s="2">
+        <v>517</v>
+      </c>
+      <c r="AL105" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM105" t="s" s="2">
         <v>518</v>
-      </c>
-      <c r="AL105" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM105" t="s" s="2">
-        <v>519</v>
       </c>
       <c r="AN105" t="s" s="2">
         <v>79</v>
@@ -14500,10 +14497,10 @@
     </row>
     <row r="106">
       <c r="A106" t="s" s="2">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B106" t="s" s="2">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" t="s" s="2">
@@ -14526,13 +14523,13 @@
         <v>79</v>
       </c>
       <c r="K106" t="s" s="2">
+        <v>520</v>
+      </c>
+      <c r="L106" t="s" s="2">
         <v>521</v>
       </c>
-      <c r="L106" t="s" s="2">
+      <c r="M106" t="s" s="2">
         <v>522</v>
-      </c>
-      <c r="M106" t="s" s="2">
-        <v>523</v>
       </c>
       <c r="N106" s="2"/>
       <c r="O106" s="2"/>
@@ -14583,7 +14580,7 @@
         <v>79</v>
       </c>
       <c r="AF106" t="s" s="2">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="AG106" t="s" s="2">
         <v>80</v>
@@ -14598,7 +14595,7 @@
         <v>102</v>
       </c>
       <c r="AK106" t="s" s="2">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="AL106" t="s" s="2">
         <v>79</v>
@@ -14615,10 +14612,10 @@
     </row>
     <row r="107">
       <c r="A107" t="s" s="2">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B107" t="s" s="2">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" t="s" s="2">
@@ -14641,23 +14638,23 @@
         <v>91</v>
       </c>
       <c r="K107" t="s" s="2">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L107" t="s" s="2">
+        <v>525</v>
+      </c>
+      <c r="M107" t="s" s="2">
         <v>526</v>
       </c>
-      <c r="M107" t="s" s="2">
+      <c r="N107" t="s" s="2">
         <v>527</v>
-      </c>
-      <c r="N107" t="s" s="2">
-        <v>528</v>
       </c>
       <c r="O107" s="2"/>
       <c r="P107" t="s" s="2">
         <v>79</v>
       </c>
       <c r="Q107" t="s" s="2">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="R107" t="s" s="2">
         <v>79</v>
@@ -14702,7 +14699,7 @@
         <v>79</v>
       </c>
       <c r="AF107" t="s" s="2">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="AG107" t="s" s="2">
         <v>80</v>
@@ -14720,7 +14717,7 @@
         <v>79</v>
       </c>
       <c r="AL107" t="s" s="2">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="AM107" t="s" s="2">
         <v>133</v>
@@ -14734,10 +14731,10 @@
     </row>
     <row r="108">
       <c r="A108" t="s" s="2">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B108" t="s" s="2">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" t="s" s="2">
@@ -14763,10 +14760,10 @@
         <v>195</v>
       </c>
       <c r="L108" t="s" s="2">
+        <v>531</v>
+      </c>
+      <c r="M108" t="s" s="2">
         <v>532</v>
-      </c>
-      <c r="M108" t="s" s="2">
-        <v>533</v>
       </c>
       <c r="N108" s="2"/>
       <c r="O108" s="2"/>
@@ -14796,11 +14793,11 @@
         <v>283</v>
       </c>
       <c r="Y108" t="s" s="2">
+        <v>533</v>
+      </c>
+      <c r="Z108" t="s" s="2">
         <v>534</v>
       </c>
-      <c r="Z108" t="s" s="2">
-        <v>535</v>
-      </c>
       <c r="AA108" t="s" s="2">
         <v>79</v>
       </c>
@@ -14817,7 +14814,7 @@
         <v>79</v>
       </c>
       <c r="AF108" t="s" s="2">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="AG108" t="s" s="2">
         <v>80</v>
@@ -14849,10 +14846,10 @@
     </row>
     <row r="109">
       <c r="A109" t="s" s="2">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B109" t="s" s="2">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="C109" s="2"/>
       <c r="D109" t="s" s="2">
@@ -14875,13 +14872,13 @@
         <v>79</v>
       </c>
       <c r="K109" t="s" s="2">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="L109" t="s" s="2">
+        <v>536</v>
+      </c>
+      <c r="M109" t="s" s="2">
         <v>537</v>
-      </c>
-      <c r="M109" t="s" s="2">
-        <v>538</v>
       </c>
       <c r="N109" s="2"/>
       <c r="O109" s="2"/>
@@ -14932,7 +14929,7 @@
         <v>79</v>
       </c>
       <c r="AF109" t="s" s="2">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="AG109" t="s" s="2">
         <v>80</v>
@@ -14944,7 +14941,7 @@
         <v>79</v>
       </c>
       <c r="AJ109" t="s" s="2">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="AK109" t="s" s="2">
         <v>79</v>
@@ -14964,10 +14961,10 @@
     </row>
     <row r="110">
       <c r="A110" t="s" s="2">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B110" t="s" s="2">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="C110" s="2"/>
       <c r="D110" t="s" s="2">
@@ -15079,10 +15076,10 @@
     </row>
     <row r="111">
       <c r="A111" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B111" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="C111" s="2"/>
       <c r="D111" t="s" s="2">
@@ -15196,14 +15193,14 @@
     </row>
     <row r="112">
       <c r="A112" t="s" s="2">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B112" t="s" s="2">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" t="s" s="2">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="E112" s="2"/>
       <c r="F112" t="s" s="2">
@@ -15225,10 +15222,10 @@
         <v>135</v>
       </c>
       <c r="L112" t="s" s="2">
+        <v>456</v>
+      </c>
+      <c r="M112" t="s" s="2">
         <v>457</v>
-      </c>
-      <c r="M112" t="s" s="2">
-        <v>458</v>
       </c>
       <c r="N112" t="s" s="2">
         <v>171</v>
@@ -15283,7 +15280,7 @@
         <v>79</v>
       </c>
       <c r="AF112" t="s" s="2">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="AG112" t="s" s="2">
         <v>80</v>
@@ -15315,10 +15312,10 @@
     </row>
     <row r="113">
       <c r="A113" t="s" s="2">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B113" t="s" s="2">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="C113" s="2"/>
       <c r="D113" t="s" s="2">
@@ -15344,10 +15341,10 @@
         <v>151</v>
       </c>
       <c r="L113" t="s" s="2">
+        <v>543</v>
+      </c>
+      <c r="M113" t="s" s="2">
         <v>544</v>
-      </c>
-      <c r="M113" t="s" s="2">
-        <v>545</v>
       </c>
       <c r="N113" s="2"/>
       <c r="O113" s="2"/>
@@ -15398,7 +15395,7 @@
         <v>79</v>
       </c>
       <c r="AF113" t="s" s="2">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="AG113" t="s" s="2">
         <v>80</v>
@@ -15416,7 +15413,7 @@
         <v>79</v>
       </c>
       <c r="AL113" t="s" s="2">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="AM113" t="s" s="2">
         <v>133</v>
@@ -15430,10 +15427,10 @@
     </row>
     <row r="114">
       <c r="A114" t="s" s="2">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="B114" t="s" s="2">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="C114" s="2"/>
       <c r="D114" t="s" s="2">
@@ -15459,10 +15456,10 @@
         <v>104</v>
       </c>
       <c r="L114" t="s" s="2">
+        <v>547</v>
+      </c>
+      <c r="M114" t="s" s="2">
         <v>548</v>
-      </c>
-      <c r="M114" t="s" s="2">
-        <v>549</v>
       </c>
       <c r="N114" s="2"/>
       <c r="O114" s="2"/>
@@ -15513,7 +15510,7 @@
         <v>79</v>
       </c>
       <c r="AF114" t="s" s="2">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="AG114" t="s" s="2">
         <v>80</v>
@@ -15545,10 +15542,10 @@
     </row>
     <row r="115">
       <c r="A115" t="s" s="2">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B115" t="s" s="2">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C115" s="2"/>
       <c r="D115" t="s" s="2">
@@ -15574,10 +15571,10 @@
         <v>338</v>
       </c>
       <c r="L115" t="s" s="2">
+        <v>550</v>
+      </c>
+      <c r="M115" t="s" s="2">
         <v>551</v>
-      </c>
-      <c r="M115" t="s" s="2">
-        <v>552</v>
       </c>
       <c r="N115" s="2"/>
       <c r="O115" s="2"/>
@@ -15628,7 +15625,7 @@
         <v>79</v>
       </c>
       <c r="AF115" t="s" s="2">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="AG115" t="s" s="2">
         <v>80</v>
@@ -15646,7 +15643,7 @@
         <v>79</v>
       </c>
       <c r="AL115" t="s" s="2">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="AM115" t="s" s="2">
         <v>133</v>
@@ -15660,10 +15657,10 @@
     </row>
     <row r="116">
       <c r="A116" t="s" s="2">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="B116" t="s" s="2">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="C116" s="2"/>
       <c r="D116" t="s" s="2">
@@ -15689,10 +15686,10 @@
         <v>338</v>
       </c>
       <c r="L116" t="s" s="2">
+        <v>554</v>
+      </c>
+      <c r="M116" t="s" s="2">
         <v>555</v>
-      </c>
-      <c r="M116" t="s" s="2">
-        <v>556</v>
       </c>
       <c r="N116" s="2"/>
       <c r="O116" s="2"/>
@@ -15743,7 +15740,7 @@
         <v>79</v>
       </c>
       <c r="AF116" t="s" s="2">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="AG116" t="s" s="2">
         <v>80</v>
@@ -15761,7 +15758,7 @@
         <v>79</v>
       </c>
       <c r="AL116" t="s" s="2">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="AM116" t="s" s="2">
         <v>133</v>
@@ -15775,10 +15772,10 @@
     </row>
     <row r="117">
       <c r="A117" t="s" s="2">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B117" t="s" s="2">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="C117" s="2"/>
       <c r="D117" t="s" s="2">
@@ -15804,10 +15801,10 @@
         <v>195</v>
       </c>
       <c r="L117" t="s" s="2">
+        <v>558</v>
+      </c>
+      <c r="M117" t="s" s="2">
         <v>559</v>
-      </c>
-      <c r="M117" t="s" s="2">
-        <v>560</v>
       </c>
       <c r="N117" s="2"/>
       <c r="O117" s="2"/>
@@ -15837,11 +15834,11 @@
         <v>283</v>
       </c>
       <c r="Y117" t="s" s="2">
+        <v>560</v>
+      </c>
+      <c r="Z117" t="s" s="2">
         <v>561</v>
       </c>
-      <c r="Z117" t="s" s="2">
-        <v>562</v>
-      </c>
       <c r="AA117" t="s" s="2">
         <v>79</v>
       </c>
@@ -15858,7 +15855,7 @@
         <v>79</v>
       </c>
       <c r="AF117" t="s" s="2">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="AG117" t="s" s="2">
         <v>80</v>
@@ -15876,7 +15873,7 @@
         <v>79</v>
       </c>
       <c r="AL117" t="s" s="2">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="AM117" t="s" s="2">
         <v>133</v>
@@ -15890,10 +15887,10 @@
     </row>
     <row r="118">
       <c r="A118" t="s" s="2">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="B118" t="s" s="2">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="C118" s="2"/>
       <c r="D118" t="s" s="2">
@@ -15919,10 +15916,10 @@
         <v>195</v>
       </c>
       <c r="L118" t="s" s="2">
+        <v>564</v>
+      </c>
+      <c r="M118" t="s" s="2">
         <v>565</v>
-      </c>
-      <c r="M118" t="s" s="2">
-        <v>566</v>
       </c>
       <c r="N118" s="2"/>
       <c r="O118" s="2"/>
@@ -15952,11 +15949,11 @@
         <v>283</v>
       </c>
       <c r="Y118" t="s" s="2">
+        <v>566</v>
+      </c>
+      <c r="Z118" t="s" s="2">
         <v>567</v>
       </c>
-      <c r="Z118" t="s" s="2">
-        <v>568</v>
-      </c>
       <c r="AA118" t="s" s="2">
         <v>79</v>
       </c>
@@ -15973,7 +15970,7 @@
         <v>79</v>
       </c>
       <c r="AF118" t="s" s="2">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="AG118" t="s" s="2">
         <v>80</v>
@@ -16005,10 +16002,10 @@
     </row>
     <row r="119">
       <c r="A119" t="s" s="2">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B119" t="s" s="2">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="C119" s="2"/>
       <c r="D119" t="s" s="2">
@@ -16031,16 +16028,16 @@
         <v>79</v>
       </c>
       <c r="K119" t="s" s="2">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="L119" t="s" s="2">
+        <v>569</v>
+      </c>
+      <c r="M119" t="s" s="2">
         <v>570</v>
       </c>
-      <c r="M119" t="s" s="2">
+      <c r="N119" t="s" s="2">
         <v>571</v>
-      </c>
-      <c r="N119" t="s" s="2">
-        <v>572</v>
       </c>
       <c r="O119" s="2"/>
       <c r="P119" t="s" s="2">
@@ -16090,7 +16087,7 @@
         <v>79</v>
       </c>
       <c r="AF119" t="s" s="2">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="AG119" t="s" s="2">
         <v>80</v>
@@ -16108,10 +16105,10 @@
         <v>79</v>
       </c>
       <c r="AL119" t="s" s="2">
+        <v>572</v>
+      </c>
+      <c r="AM119" t="s" s="2">
         <v>573</v>
-      </c>
-      <c r="AM119" t="s" s="2">
-        <v>574</v>
       </c>
       <c r="AN119" t="s" s="2">
         <v>79</v>
@@ -16122,10 +16119,10 @@
     </row>
     <row r="120">
       <c r="A120" t="s" s="2">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="B120" t="s" s="2">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="C120" s="2"/>
       <c r="D120" t="s" s="2">
@@ -16237,10 +16234,10 @@
     </row>
     <row r="121">
       <c r="A121" t="s" s="2">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="B121" t="s" s="2">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="C121" s="2"/>
       <c r="D121" t="s" s="2">
@@ -16354,14 +16351,14 @@
     </row>
     <row r="122">
       <c r="A122" t="s" s="2">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="B122" t="s" s="2">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C122" s="2"/>
       <c r="D122" t="s" s="2">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="E122" s="2"/>
       <c r="F122" t="s" s="2">
@@ -16383,10 +16380,10 @@
         <v>135</v>
       </c>
       <c r="L122" t="s" s="2">
+        <v>456</v>
+      </c>
+      <c r="M122" t="s" s="2">
         <v>457</v>
-      </c>
-      <c r="M122" t="s" s="2">
-        <v>458</v>
       </c>
       <c r="N122" t="s" s="2">
         <v>171</v>
@@ -16441,7 +16438,7 @@
         <v>79</v>
       </c>
       <c r="AF122" t="s" s="2">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="AG122" t="s" s="2">
         <v>80</v>
@@ -16473,10 +16470,10 @@
     </row>
     <row r="123">
       <c r="A123" t="s" s="2">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="B123" t="s" s="2">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C123" s="2"/>
       <c r="D123" t="s" s="2">
@@ -16502,10 +16499,10 @@
         <v>338</v>
       </c>
       <c r="L123" t="s" s="2">
+        <v>578</v>
+      </c>
+      <c r="M123" t="s" s="2">
         <v>579</v>
-      </c>
-      <c r="M123" t="s" s="2">
-        <v>580</v>
       </c>
       <c r="N123" s="2"/>
       <c r="O123" s="2"/>
@@ -16556,7 +16553,7 @@
         <v>79</v>
       </c>
       <c r="AF123" t="s" s="2">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AG123" t="s" s="2">
         <v>80</v>
@@ -16574,7 +16571,7 @@
         <v>79</v>
       </c>
       <c r="AL123" t="s" s="2">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="AM123" t="s" s="2">
         <v>346</v>
@@ -16588,10 +16585,10 @@
     </row>
     <row r="124">
       <c r="A124" t="s" s="2">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="B124" t="s" s="2">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="C124" s="2"/>
       <c r="D124" t="s" s="2">
@@ -16614,13 +16611,13 @@
         <v>79</v>
       </c>
       <c r="K124" t="s" s="2">
+        <v>582</v>
+      </c>
+      <c r="L124" t="s" s="2">
         <v>583</v>
       </c>
-      <c r="L124" t="s" s="2">
+      <c r="M124" t="s" s="2">
         <v>584</v>
-      </c>
-      <c r="M124" t="s" s="2">
-        <v>585</v>
       </c>
       <c r="N124" s="2"/>
       <c r="O124" s="2"/>
@@ -16671,7 +16668,7 @@
         <v>79</v>
       </c>
       <c r="AF124" t="s" s="2">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="AG124" t="s" s="2">
         <v>80</v>
@@ -16689,10 +16686,10 @@
         <v>79</v>
       </c>
       <c r="AL124" t="s" s="2">
+        <v>585</v>
+      </c>
+      <c r="AM124" t="s" s="2">
         <v>586</v>
-      </c>
-      <c r="AM124" t="s" s="2">
-        <v>587</v>
       </c>
       <c r="AN124" t="s" s="2">
         <v>79</v>
@@ -16703,10 +16700,10 @@
     </row>
     <row r="125">
       <c r="A125" t="s" s="2">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B125" t="s" s="2">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="C125" s="2"/>
       <c r="D125" t="s" s="2">
@@ -16729,13 +16726,13 @@
         <v>79</v>
       </c>
       <c r="K125" t="s" s="2">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L125" t="s" s="2">
+        <v>588</v>
+      </c>
+      <c r="M125" t="s" s="2">
         <v>589</v>
-      </c>
-      <c r="M125" t="s" s="2">
-        <v>590</v>
       </c>
       <c r="N125" s="2"/>
       <c r="O125" s="2"/>
@@ -16786,7 +16783,7 @@
         <v>79</v>
       </c>
       <c r="AF125" t="s" s="2">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="AG125" t="s" s="2">
         <v>80</v>
@@ -16804,10 +16801,10 @@
         <v>79</v>
       </c>
       <c r="AL125" t="s" s="2">
+        <v>590</v>
+      </c>
+      <c r="AM125" t="s" s="2">
         <v>591</v>
-      </c>
-      <c r="AM125" t="s" s="2">
-        <v>592</v>
       </c>
       <c r="AN125" t="s" s="2">
         <v>79</v>
@@ -16818,10 +16815,10 @@
     </row>
     <row r="126">
       <c r="A126" t="s" s="2">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="B126" t="s" s="2">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C126" s="2"/>
       <c r="D126" t="s" s="2">
@@ -16844,13 +16841,13 @@
         <v>79</v>
       </c>
       <c r="K126" t="s" s="2">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="L126" t="s" s="2">
+        <v>593</v>
+      </c>
+      <c r="M126" t="s" s="2">
         <v>594</v>
-      </c>
-      <c r="M126" t="s" s="2">
-        <v>595</v>
       </c>
       <c r="N126" s="2"/>
       <c r="O126" s="2"/>
@@ -16901,7 +16898,7 @@
         <v>79</v>
       </c>
       <c r="AF126" t="s" s="2">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="AG126" t="s" s="2">
         <v>80</v>
@@ -16933,10 +16930,10 @@
     </row>
     <row r="127">
       <c r="A127" t="s" s="2">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B127" t="s" s="2">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="C127" s="2"/>
       <c r="D127" t="s" s="2">
@@ -17048,10 +17045,10 @@
     </row>
     <row r="128">
       <c r="A128" t="s" s="2">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B128" t="s" s="2">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="C128" s="2"/>
       <c r="D128" t="s" s="2">
@@ -17165,14 +17162,14 @@
     </row>
     <row r="129">
       <c r="A129" t="s" s="2">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B129" t="s" s="2">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="C129" s="2"/>
       <c r="D129" t="s" s="2">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="E129" s="2"/>
       <c r="F129" t="s" s="2">
@@ -17194,10 +17191,10 @@
         <v>135</v>
       </c>
       <c r="L129" t="s" s="2">
+        <v>456</v>
+      </c>
+      <c r="M129" t="s" s="2">
         <v>457</v>
-      </c>
-      <c r="M129" t="s" s="2">
-        <v>458</v>
       </c>
       <c r="N129" t="s" s="2">
         <v>171</v>
@@ -17252,7 +17249,7 @@
         <v>79</v>
       </c>
       <c r="AF129" t="s" s="2">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="AG129" t="s" s="2">
         <v>80</v>
@@ -17284,10 +17281,10 @@
     </row>
     <row r="130">
       <c r="A130" t="s" s="2">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B130" t="s" s="2">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="C130" s="2"/>
       <c r="D130" t="s" s="2">
@@ -17313,10 +17310,10 @@
         <v>151</v>
       </c>
       <c r="L130" t="s" s="2">
+        <v>599</v>
+      </c>
+      <c r="M130" t="s" s="2">
         <v>600</v>
-      </c>
-      <c r="M130" t="s" s="2">
-        <v>601</v>
       </c>
       <c r="N130" s="2"/>
       <c r="O130" s="2"/>
@@ -17347,7 +17344,7 @@
       </c>
       <c r="Y130" s="2"/>
       <c r="Z130" t="s" s="2">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="AA130" t="s" s="2">
         <v>79</v>
@@ -17365,7 +17362,7 @@
         <v>79</v>
       </c>
       <c r="AF130" t="s" s="2">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="AG130" t="s" s="2">
         <v>80</v>
@@ -17397,10 +17394,10 @@
     </row>
     <row r="131">
       <c r="A131" t="s" s="2">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B131" t="s" s="2">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="C131" s="2"/>
       <c r="D131" t="s" s="2">
@@ -17423,13 +17420,13 @@
         <v>79</v>
       </c>
       <c r="K131" t="s" s="2">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="L131" t="s" s="2">
+        <v>603</v>
+      </c>
+      <c r="M131" t="s" s="2">
         <v>604</v>
-      </c>
-      <c r="M131" t="s" s="2">
-        <v>605</v>
       </c>
       <c r="N131" s="2"/>
       <c r="O131" s="2"/>
@@ -17480,7 +17477,7 @@
         <v>79</v>
       </c>
       <c r="AF131" t="s" s="2">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="AG131" t="s" s="2">
         <v>80</v>
@@ -17512,10 +17509,10 @@
     </row>
     <row r="132">
       <c r="A132" t="s" s="2">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B132" t="s" s="2">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C132" s="2"/>
       <c r="D132" t="s" s="2">
@@ -17541,10 +17538,10 @@
         <v>195</v>
       </c>
       <c r="L132" t="s" s="2">
+        <v>606</v>
+      </c>
+      <c r="M132" t="s" s="2">
         <v>607</v>
-      </c>
-      <c r="M132" t="s" s="2">
-        <v>608</v>
       </c>
       <c r="N132" s="2"/>
       <c r="O132" s="2"/>
@@ -17574,11 +17571,11 @@
         <v>114</v>
       </c>
       <c r="Y132" t="s" s="2">
+        <v>608</v>
+      </c>
+      <c r="Z132" t="s" s="2">
         <v>609</v>
       </c>
-      <c r="Z132" t="s" s="2">
-        <v>610</v>
-      </c>
       <c r="AA132" t="s" s="2">
         <v>79</v>
       </c>
@@ -17595,7 +17592,7 @@
         <v>79</v>
       </c>
       <c r="AF132" t="s" s="2">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="AG132" t="s" s="2">
         <v>80</v>
@@ -17627,10 +17624,10 @@
     </row>
     <row r="133">
       <c r="A133" t="s" s="2">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B133" t="s" s="2">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="C133" s="2"/>
       <c r="D133" t="s" s="2">
@@ -17653,16 +17650,16 @@
         <v>79</v>
       </c>
       <c r="K133" t="s" s="2">
+        <v>611</v>
+      </c>
+      <c r="L133" t="s" s="2">
         <v>612</v>
       </c>
-      <c r="L133" t="s" s="2">
+      <c r="M133" t="s" s="2">
         <v>613</v>
       </c>
-      <c r="M133" t="s" s="2">
+      <c r="N133" t="s" s="2">
         <v>614</v>
-      </c>
-      <c r="N133" t="s" s="2">
-        <v>615</v>
       </c>
       <c r="O133" s="2"/>
       <c r="P133" t="s" s="2">
@@ -17710,7 +17707,7 @@
         <v>139</v>
       </c>
       <c r="AF133" t="s" s="2">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="AG133" t="s" s="2">
         <v>90</v>
@@ -17742,13 +17739,13 @@
     </row>
     <row r="134">
       <c r="A134" t="s" s="2">
+        <v>615</v>
+      </c>
+      <c r="B134" t="s" s="2">
+        <v>610</v>
+      </c>
+      <c r="C134" t="s" s="2">
         <v>616</v>
-      </c>
-      <c r="B134" t="s" s="2">
-        <v>611</v>
-      </c>
-      <c r="C134" t="s" s="2">
-        <v>617</v>
       </c>
       <c r="D134" t="s" s="2">
         <v>79</v>
@@ -17770,16 +17767,16 @@
         <v>79</v>
       </c>
       <c r="K134" t="s" s="2">
+        <v>617</v>
+      </c>
+      <c r="L134" t="s" s="2">
         <v>618</v>
       </c>
-      <c r="L134" t="s" s="2">
-        <v>619</v>
-      </c>
       <c r="M134" t="s" s="2">
+        <v>613</v>
+      </c>
+      <c r="N134" t="s" s="2">
         <v>614</v>
-      </c>
-      <c r="N134" t="s" s="2">
-        <v>615</v>
       </c>
       <c r="O134" s="2"/>
       <c r="P134" t="s" s="2">
@@ -17829,7 +17826,7 @@
         <v>79</v>
       </c>
       <c r="AF134" t="s" s="2">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="AG134" t="s" s="2">
         <v>90</v>
@@ -17861,10 +17858,10 @@
     </row>
     <row r="135">
       <c r="A135" t="s" s="2">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B135" t="s" s="2">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="C135" s="2"/>
       <c r="D135" t="s" s="2">
@@ -17887,16 +17884,16 @@
         <v>79</v>
       </c>
       <c r="K135" t="s" s="2">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="L135" t="s" s="2">
+        <v>620</v>
+      </c>
+      <c r="M135" t="s" s="2">
         <v>621</v>
       </c>
-      <c r="M135" t="s" s="2">
-        <v>622</v>
-      </c>
       <c r="N135" t="s" s="2">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="O135" s="2"/>
       <c r="P135" t="s" s="2">
@@ -17946,7 +17943,7 @@
         <v>79</v>
       </c>
       <c r="AF135" t="s" s="2">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="AG135" t="s" s="2">
         <v>80</v>

</xml_diff>

<commit_message>
fix: supprime la ligne ^short "Commentaire" résiduelle sur note 1858d35db62b68742c8e0afc347bc08771c5955f
</commit_message>
<xml_diff>
--- a/nr-doc-core-immunization/ig/StructureDefinition-fr-core-immunization.xlsx
+++ b/nr-doc-core-immunization/ig/StructureDefinition-fr-core-immunization.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-29T15:19:05+00:00</t>
+    <t>2026-07-20T14:29:12+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1339,7 +1339,7 @@
     <t>Body site where vaccine was administered.</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-immunization-approach-site-code-cisis|20260420150249</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-immunization-approach-site-code-cisis|20260619134041</t>
   </si>
   <si>
     <t>RXR-2</t>
@@ -1360,7 +1360,7 @@
     <t>The path by which the vaccine product is taken into the body.</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-immunization-route-code-cisis|20260420150250</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-immunization-route-code-cisis|20260619134042</t>
   </si>
   <si>
     <t>RXR-1</t>
@@ -1532,7 +1532,7 @@
 </t>
   </si>
   <si>
-    <t>Commentaire</t>
+    <t>Additional immunization notes</t>
   </si>
   <si>
     <t>Extra information about the immunization that is not conveyed by the other attributes.</t>
@@ -1879,7 +1879,7 @@
     <t>One possible path to achieve presumed immunity against a disease - within the context of an authority.</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-hl7-v3-ActSubstanceAdministrationImmunizationCode-cisis|20260420150251</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-hl7-v3-ActSubstanceAdministrationImmunizationCode-cisis|20260619134043</t>
   </si>
   <si>
     <t>Immunization.protocolApplied.authority</t>
@@ -13702,7 +13702,7 @@
         <v>80</v>
       </c>
       <c r="G99" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="H99" t="s" s="2">
         <v>79</v>

</xml_diff>